<commit_message>
Party size: +1s and children seated and checked in together
New Guest has Party size; the Excel import and template read a Party Size column. Companions are created as "First Last +1", "+2"… at the same table (Setting party:<event>:<guest>). Checking in the main guest (desk, table card or their phone) checks in the whole party; history notes it.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LYD99kSvVYUTkYKht9B4pf
</commit_message>
<xml_diff>
--- a/public/templates/Seating4U-guest-template.xlsx
+++ b/public/templates/Seating4U-guest-template.xlsx
@@ -249,6 +249,11 @@
     <comment ref="G1" authorId="0" shapeId="0">
       <text>
         <t>Optional. A note for the desk. With a note, the guest's phone won't show the seat; the desk reads the note and must write a desk note before giving the seat.</t>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional. How many people in total, including this guest (e.g. 3 = guest + 2). They get seats at the same table and are checked in together. Leave empty for 1.</t>
       </text>
     </comment>
   </commentList>
@@ -544,7 +549,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G501"/>
+  <dimension ref="A1:H501"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="1" min="1" max="1"/>
@@ -554,7 +559,7 @@
     <col width="18" customWidth="1" style="1" min="5" max="5"/>
     <col width="8" customWidth="1" style="1" min="6" max="6"/>
     <col width="40" customWidth="1" style="1" min="7" max="7"/>
-    <col width="13" customWidth="1" style="1" min="8" max="8"/>
+    <col width="11" customWidth="1" style="1" min="8" max="8"/>
     <col width="13" customWidth="1" style="1" min="9" max="9"/>
     <col width="13" customWidth="1" style="1" min="10" max="10"/>
     <col width="13" customWidth="1" style="1" min="11" max="11"/>
@@ -611,6 +616,11 @@
           <t>Note</t>
         </is>
       </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>Party Size</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="n"/>
@@ -620,6 +630,7 @@
       <c r="E2" s="4" t="n"/>
       <c r="F2" s="4" t="n"/>
       <c r="G2" s="4" t="n"/>
+      <c r="H2" s="4" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n"/>
@@ -629,6 +640,7 @@
       <c r="E3" s="4" t="n"/>
       <c r="F3" s="4" t="n"/>
       <c r="G3" s="4" t="n"/>
+      <c r="H3" s="4" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n"/>
@@ -638,6 +650,7 @@
       <c r="E4" s="4" t="n"/>
       <c r="F4" s="4" t="n"/>
       <c r="G4" s="4" t="n"/>
+      <c r="H4" s="4" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n"/>
@@ -647,6 +660,7 @@
       <c r="E5" s="4" t="n"/>
       <c r="F5" s="4" t="n"/>
       <c r="G5" s="4" t="n"/>
+      <c r="H5" s="4" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n"/>
@@ -656,6 +670,7 @@
       <c r="E6" s="4" t="n"/>
       <c r="F6" s="4" t="n"/>
       <c r="G6" s="4" t="n"/>
+      <c r="H6" s="4" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n"/>
@@ -665,6 +680,7 @@
       <c r="E7" s="4" t="n"/>
       <c r="F7" s="4" t="n"/>
       <c r="G7" s="4" t="n"/>
+      <c r="H7" s="4" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n"/>
@@ -674,6 +690,7 @@
       <c r="E8" s="4" t="n"/>
       <c r="F8" s="4" t="n"/>
       <c r="G8" s="4" t="n"/>
+      <c r="H8" s="4" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n"/>
@@ -683,6 +700,7 @@
       <c r="E9" s="4" t="n"/>
       <c r="F9" s="4" t="n"/>
       <c r="G9" s="4" t="n"/>
+      <c r="H9" s="4" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n"/>
@@ -692,6 +710,7 @@
       <c r="E10" s="4" t="n"/>
       <c r="F10" s="4" t="n"/>
       <c r="G10" s="4" t="n"/>
+      <c r="H10" s="4" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n"/>
@@ -701,6 +720,7 @@
       <c r="E11" s="4" t="n"/>
       <c r="F11" s="4" t="n"/>
       <c r="G11" s="4" t="n"/>
+      <c r="H11" s="4" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n"/>
@@ -710,6 +730,7 @@
       <c r="E12" s="4" t="n"/>
       <c r="F12" s="4" t="n"/>
       <c r="G12" s="4" t="n"/>
+      <c r="H12" s="4" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n"/>
@@ -719,6 +740,7 @@
       <c r="E13" s="4" t="n"/>
       <c r="F13" s="4" t="n"/>
       <c r="G13" s="4" t="n"/>
+      <c r="H13" s="4" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n"/>
@@ -728,6 +750,7 @@
       <c r="E14" s="4" t="n"/>
       <c r="F14" s="4" t="n"/>
       <c r="G14" s="4" t="n"/>
+      <c r="H14" s="4" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n"/>
@@ -737,6 +760,7 @@
       <c r="E15" s="4" t="n"/>
       <c r="F15" s="4" t="n"/>
       <c r="G15" s="4" t="n"/>
+      <c r="H15" s="4" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n"/>
@@ -746,6 +770,7 @@
       <c r="E16" s="4" t="n"/>
       <c r="F16" s="4" t="n"/>
       <c r="G16" s="4" t="n"/>
+      <c r="H16" s="4" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n"/>
@@ -755,6 +780,7 @@
       <c r="E17" s="4" t="n"/>
       <c r="F17" s="4" t="n"/>
       <c r="G17" s="4" t="n"/>
+      <c r="H17" s="4" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n"/>
@@ -764,6 +790,7 @@
       <c r="E18" s="4" t="n"/>
       <c r="F18" s="4" t="n"/>
       <c r="G18" s="4" t="n"/>
+      <c r="H18" s="4" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n"/>
@@ -773,6 +800,7 @@
       <c r="E19" s="4" t="n"/>
       <c r="F19" s="4" t="n"/>
       <c r="G19" s="4" t="n"/>
+      <c r="H19" s="4" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n"/>
@@ -782,6 +810,7 @@
       <c r="E20" s="4" t="n"/>
       <c r="F20" s="4" t="n"/>
       <c r="G20" s="4" t="n"/>
+      <c r="H20" s="4" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n"/>
@@ -791,6 +820,7 @@
       <c r="E21" s="4" t="n"/>
       <c r="F21" s="4" t="n"/>
       <c r="G21" s="4" t="n"/>
+      <c r="H21" s="4" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n"/>
@@ -800,6 +830,7 @@
       <c r="E22" s="4" t="n"/>
       <c r="F22" s="4" t="n"/>
       <c r="G22" s="4" t="n"/>
+      <c r="H22" s="4" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n"/>
@@ -809,6 +840,7 @@
       <c r="E23" s="4" t="n"/>
       <c r="F23" s="4" t="n"/>
       <c r="G23" s="4" t="n"/>
+      <c r="H23" s="4" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n"/>
@@ -818,6 +850,7 @@
       <c r="E24" s="4" t="n"/>
       <c r="F24" s="4" t="n"/>
       <c r="G24" s="4" t="n"/>
+      <c r="H24" s="4" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n"/>
@@ -827,6 +860,7 @@
       <c r="E25" s="4" t="n"/>
       <c r="F25" s="4" t="n"/>
       <c r="G25" s="4" t="n"/>
+      <c r="H25" s="4" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="4" t="n"/>
@@ -836,6 +870,7 @@
       <c r="E26" s="4" t="n"/>
       <c r="F26" s="4" t="n"/>
       <c r="G26" s="4" t="n"/>
+      <c r="H26" s="4" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n"/>
@@ -845,6 +880,7 @@
       <c r="E27" s="4" t="n"/>
       <c r="F27" s="4" t="n"/>
       <c r="G27" s="4" t="n"/>
+      <c r="H27" s="4" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="4" t="n"/>
@@ -854,6 +890,7 @@
       <c r="E28" s="4" t="n"/>
       <c r="F28" s="4" t="n"/>
       <c r="G28" s="4" t="n"/>
+      <c r="H28" s="4" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="4" t="n"/>
@@ -863,6 +900,7 @@
       <c r="E29" s="4" t="n"/>
       <c r="F29" s="4" t="n"/>
       <c r="G29" s="4" t="n"/>
+      <c r="H29" s="4" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="4" t="n"/>
@@ -872,6 +910,7 @@
       <c r="E30" s="4" t="n"/>
       <c r="F30" s="4" t="n"/>
       <c r="G30" s="4" t="n"/>
+      <c r="H30" s="4" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="4" t="n"/>
@@ -881,6 +920,7 @@
       <c r="E31" s="4" t="n"/>
       <c r="F31" s="4" t="n"/>
       <c r="G31" s="4" t="n"/>
+      <c r="H31" s="4" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="4" t="n"/>
@@ -890,6 +930,7 @@
       <c r="E32" s="4" t="n"/>
       <c r="F32" s="4" t="n"/>
       <c r="G32" s="4" t="n"/>
+      <c r="H32" s="4" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="n"/>
@@ -899,6 +940,7 @@
       <c r="E33" s="4" t="n"/>
       <c r="F33" s="4" t="n"/>
       <c r="G33" s="4" t="n"/>
+      <c r="H33" s="4" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="4" t="n"/>
@@ -908,6 +950,7 @@
       <c r="E34" s="4" t="n"/>
       <c r="F34" s="4" t="n"/>
       <c r="G34" s="4" t="n"/>
+      <c r="H34" s="4" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="4" t="n"/>
@@ -917,6 +960,7 @@
       <c r="E35" s="4" t="n"/>
       <c r="F35" s="4" t="n"/>
       <c r="G35" s="4" t="n"/>
+      <c r="H35" s="4" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="4" t="n"/>
@@ -926,6 +970,7 @@
       <c r="E36" s="4" t="n"/>
       <c r="F36" s="4" t="n"/>
       <c r="G36" s="4" t="n"/>
+      <c r="H36" s="4" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="4" t="n"/>
@@ -935,6 +980,7 @@
       <c r="E37" s="4" t="n"/>
       <c r="F37" s="4" t="n"/>
       <c r="G37" s="4" t="n"/>
+      <c r="H37" s="4" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="4" t="n"/>
@@ -944,6 +990,7 @@
       <c r="E38" s="4" t="n"/>
       <c r="F38" s="4" t="n"/>
       <c r="G38" s="4" t="n"/>
+      <c r="H38" s="4" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="4" t="n"/>
@@ -953,6 +1000,7 @@
       <c r="E39" s="4" t="n"/>
       <c r="F39" s="4" t="n"/>
       <c r="G39" s="4" t="n"/>
+      <c r="H39" s="4" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="4" t="n"/>
@@ -962,6 +1010,7 @@
       <c r="E40" s="4" t="n"/>
       <c r="F40" s="4" t="n"/>
       <c r="G40" s="4" t="n"/>
+      <c r="H40" s="4" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="4" t="n"/>
@@ -971,6 +1020,7 @@
       <c r="E41" s="4" t="n"/>
       <c r="F41" s="4" t="n"/>
       <c r="G41" s="4" t="n"/>
+      <c r="H41" s="4" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="4" t="n"/>
@@ -980,6 +1030,7 @@
       <c r="E42" s="4" t="n"/>
       <c r="F42" s="4" t="n"/>
       <c r="G42" s="4" t="n"/>
+      <c r="H42" s="4" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="4" t="n"/>
@@ -989,6 +1040,7 @@
       <c r="E43" s="4" t="n"/>
       <c r="F43" s="4" t="n"/>
       <c r="G43" s="4" t="n"/>
+      <c r="H43" s="4" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="4" t="n"/>
@@ -998,6 +1050,7 @@
       <c r="E44" s="4" t="n"/>
       <c r="F44" s="4" t="n"/>
       <c r="G44" s="4" t="n"/>
+      <c r="H44" s="4" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="4" t="n"/>
@@ -1007,6 +1060,7 @@
       <c r="E45" s="4" t="n"/>
       <c r="F45" s="4" t="n"/>
       <c r="G45" s="4" t="n"/>
+      <c r="H45" s="4" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="4" t="n"/>
@@ -1016,6 +1070,7 @@
       <c r="E46" s="4" t="n"/>
       <c r="F46" s="4" t="n"/>
       <c r="G46" s="4" t="n"/>
+      <c r="H46" s="4" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="4" t="n"/>
@@ -1025,6 +1080,7 @@
       <c r="E47" s="4" t="n"/>
       <c r="F47" s="4" t="n"/>
       <c r="G47" s="4" t="n"/>
+      <c r="H47" s="4" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="4" t="n"/>
@@ -1034,6 +1090,7 @@
       <c r="E48" s="4" t="n"/>
       <c r="F48" s="4" t="n"/>
       <c r="G48" s="4" t="n"/>
+      <c r="H48" s="4" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="4" t="n"/>
@@ -1043,6 +1100,7 @@
       <c r="E49" s="4" t="n"/>
       <c r="F49" s="4" t="n"/>
       <c r="G49" s="4" t="n"/>
+      <c r="H49" s="4" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="4" t="n"/>
@@ -1052,6 +1110,7 @@
       <c r="E50" s="4" t="n"/>
       <c r="F50" s="4" t="n"/>
       <c r="G50" s="4" t="n"/>
+      <c r="H50" s="4" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="4" t="n"/>
@@ -1061,6 +1120,7 @@
       <c r="E51" s="4" t="n"/>
       <c r="F51" s="4" t="n"/>
       <c r="G51" s="4" t="n"/>
+      <c r="H51" s="4" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="4" t="n"/>
@@ -1070,6 +1130,7 @@
       <c r="E52" s="4" t="n"/>
       <c r="F52" s="4" t="n"/>
       <c r="G52" s="4" t="n"/>
+      <c r="H52" s="4" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="4" t="n"/>
@@ -1079,6 +1140,7 @@
       <c r="E53" s="4" t="n"/>
       <c r="F53" s="4" t="n"/>
       <c r="G53" s="4" t="n"/>
+      <c r="H53" s="4" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="4" t="n"/>
@@ -1088,6 +1150,7 @@
       <c r="E54" s="4" t="n"/>
       <c r="F54" s="4" t="n"/>
       <c r="G54" s="4" t="n"/>
+      <c r="H54" s="4" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="4" t="n"/>
@@ -1097,6 +1160,7 @@
       <c r="E55" s="4" t="n"/>
       <c r="F55" s="4" t="n"/>
       <c r="G55" s="4" t="n"/>
+      <c r="H55" s="4" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="4" t="n"/>
@@ -1106,6 +1170,7 @@
       <c r="E56" s="4" t="n"/>
       <c r="F56" s="4" t="n"/>
       <c r="G56" s="4" t="n"/>
+      <c r="H56" s="4" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="4" t="n"/>
@@ -1115,6 +1180,7 @@
       <c r="E57" s="4" t="n"/>
       <c r="F57" s="4" t="n"/>
       <c r="G57" s="4" t="n"/>
+      <c r="H57" s="4" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="4" t="n"/>
@@ -1124,6 +1190,7 @@
       <c r="E58" s="4" t="n"/>
       <c r="F58" s="4" t="n"/>
       <c r="G58" s="4" t="n"/>
+      <c r="H58" s="4" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="4" t="n"/>
@@ -1133,6 +1200,7 @@
       <c r="E59" s="4" t="n"/>
       <c r="F59" s="4" t="n"/>
       <c r="G59" s="4" t="n"/>
+      <c r="H59" s="4" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="4" t="n"/>
@@ -1142,6 +1210,7 @@
       <c r="E60" s="4" t="n"/>
       <c r="F60" s="4" t="n"/>
       <c r="G60" s="4" t="n"/>
+      <c r="H60" s="4" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="4" t="n"/>
@@ -1151,6 +1220,7 @@
       <c r="E61" s="4" t="n"/>
       <c r="F61" s="4" t="n"/>
       <c r="G61" s="4" t="n"/>
+      <c r="H61" s="4" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="4" t="n"/>
@@ -1160,6 +1230,7 @@
       <c r="E62" s="4" t="n"/>
       <c r="F62" s="4" t="n"/>
       <c r="G62" s="4" t="n"/>
+      <c r="H62" s="4" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="4" t="n"/>
@@ -1169,6 +1240,7 @@
       <c r="E63" s="4" t="n"/>
       <c r="F63" s="4" t="n"/>
       <c r="G63" s="4" t="n"/>
+      <c r="H63" s="4" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="4" t="n"/>
@@ -1178,6 +1250,7 @@
       <c r="E64" s="4" t="n"/>
       <c r="F64" s="4" t="n"/>
       <c r="G64" s="4" t="n"/>
+      <c r="H64" s="4" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="4" t="n"/>
@@ -1187,6 +1260,7 @@
       <c r="E65" s="4" t="n"/>
       <c r="F65" s="4" t="n"/>
       <c r="G65" s="4" t="n"/>
+      <c r="H65" s="4" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="4" t="n"/>
@@ -1196,6 +1270,7 @@
       <c r="E66" s="4" t="n"/>
       <c r="F66" s="4" t="n"/>
       <c r="G66" s="4" t="n"/>
+      <c r="H66" s="4" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="4" t="n"/>
@@ -1205,6 +1280,7 @@
       <c r="E67" s="4" t="n"/>
       <c r="F67" s="4" t="n"/>
       <c r="G67" s="4" t="n"/>
+      <c r="H67" s="4" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="4" t="n"/>
@@ -1214,6 +1290,7 @@
       <c r="E68" s="4" t="n"/>
       <c r="F68" s="4" t="n"/>
       <c r="G68" s="4" t="n"/>
+      <c r="H68" s="4" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="4" t="n"/>
@@ -1223,6 +1300,7 @@
       <c r="E69" s="4" t="n"/>
       <c r="F69" s="4" t="n"/>
       <c r="G69" s="4" t="n"/>
+      <c r="H69" s="4" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="4" t="n"/>
@@ -1232,6 +1310,7 @@
       <c r="E70" s="4" t="n"/>
       <c r="F70" s="4" t="n"/>
       <c r="G70" s="4" t="n"/>
+      <c r="H70" s="4" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="4" t="n"/>
@@ -1241,6 +1320,7 @@
       <c r="E71" s="4" t="n"/>
       <c r="F71" s="4" t="n"/>
       <c r="G71" s="4" t="n"/>
+      <c r="H71" s="4" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="4" t="n"/>
@@ -1250,6 +1330,7 @@
       <c r="E72" s="4" t="n"/>
       <c r="F72" s="4" t="n"/>
       <c r="G72" s="4" t="n"/>
+      <c r="H72" s="4" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="4" t="n"/>
@@ -1259,6 +1340,7 @@
       <c r="E73" s="4" t="n"/>
       <c r="F73" s="4" t="n"/>
       <c r="G73" s="4" t="n"/>
+      <c r="H73" s="4" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="4" t="n"/>
@@ -1268,6 +1350,7 @@
       <c r="E74" s="4" t="n"/>
       <c r="F74" s="4" t="n"/>
       <c r="G74" s="4" t="n"/>
+      <c r="H74" s="4" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="4" t="n"/>
@@ -1277,6 +1360,7 @@
       <c r="E75" s="4" t="n"/>
       <c r="F75" s="4" t="n"/>
       <c r="G75" s="4" t="n"/>
+      <c r="H75" s="4" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="4" t="n"/>
@@ -1286,6 +1370,7 @@
       <c r="E76" s="4" t="n"/>
       <c r="F76" s="4" t="n"/>
       <c r="G76" s="4" t="n"/>
+      <c r="H76" s="4" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="4" t="n"/>
@@ -1295,6 +1380,7 @@
       <c r="E77" s="4" t="n"/>
       <c r="F77" s="4" t="n"/>
       <c r="G77" s="4" t="n"/>
+      <c r="H77" s="4" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="4" t="n"/>
@@ -1304,6 +1390,7 @@
       <c r="E78" s="4" t="n"/>
       <c r="F78" s="4" t="n"/>
       <c r="G78" s="4" t="n"/>
+      <c r="H78" s="4" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="4" t="n"/>
@@ -1313,6 +1400,7 @@
       <c r="E79" s="4" t="n"/>
       <c r="F79" s="4" t="n"/>
       <c r="G79" s="4" t="n"/>
+      <c r="H79" s="4" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="4" t="n"/>
@@ -1322,6 +1410,7 @@
       <c r="E80" s="4" t="n"/>
       <c r="F80" s="4" t="n"/>
       <c r="G80" s="4" t="n"/>
+      <c r="H80" s="4" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="4" t="n"/>
@@ -1331,6 +1420,7 @@
       <c r="E81" s="4" t="n"/>
       <c r="F81" s="4" t="n"/>
       <c r="G81" s="4" t="n"/>
+      <c r="H81" s="4" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="4" t="n"/>
@@ -1340,6 +1430,7 @@
       <c r="E82" s="4" t="n"/>
       <c r="F82" s="4" t="n"/>
       <c r="G82" s="4" t="n"/>
+      <c r="H82" s="4" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="4" t="n"/>
@@ -1349,6 +1440,7 @@
       <c r="E83" s="4" t="n"/>
       <c r="F83" s="4" t="n"/>
       <c r="G83" s="4" t="n"/>
+      <c r="H83" s="4" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="4" t="n"/>
@@ -1358,6 +1450,7 @@
       <c r="E84" s="4" t="n"/>
       <c r="F84" s="4" t="n"/>
       <c r="G84" s="4" t="n"/>
+      <c r="H84" s="4" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="4" t="n"/>
@@ -1367,6 +1460,7 @@
       <c r="E85" s="4" t="n"/>
       <c r="F85" s="4" t="n"/>
       <c r="G85" s="4" t="n"/>
+      <c r="H85" s="4" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="4" t="n"/>
@@ -1376,6 +1470,7 @@
       <c r="E86" s="4" t="n"/>
       <c r="F86" s="4" t="n"/>
       <c r="G86" s="4" t="n"/>
+      <c r="H86" s="4" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="4" t="n"/>
@@ -1385,6 +1480,7 @@
       <c r="E87" s="4" t="n"/>
       <c r="F87" s="4" t="n"/>
       <c r="G87" s="4" t="n"/>
+      <c r="H87" s="4" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="4" t="n"/>
@@ -1394,6 +1490,7 @@
       <c r="E88" s="4" t="n"/>
       <c r="F88" s="4" t="n"/>
       <c r="G88" s="4" t="n"/>
+      <c r="H88" s="4" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="4" t="n"/>
@@ -1403,6 +1500,7 @@
       <c r="E89" s="4" t="n"/>
       <c r="F89" s="4" t="n"/>
       <c r="G89" s="4" t="n"/>
+      <c r="H89" s="4" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="4" t="n"/>
@@ -1412,6 +1510,7 @@
       <c r="E90" s="4" t="n"/>
       <c r="F90" s="4" t="n"/>
       <c r="G90" s="4" t="n"/>
+      <c r="H90" s="4" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="4" t="n"/>
@@ -1421,6 +1520,7 @@
       <c r="E91" s="4" t="n"/>
       <c r="F91" s="4" t="n"/>
       <c r="G91" s="4" t="n"/>
+      <c r="H91" s="4" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="4" t="n"/>
@@ -1430,6 +1530,7 @@
       <c r="E92" s="4" t="n"/>
       <c r="F92" s="4" t="n"/>
       <c r="G92" s="4" t="n"/>
+      <c r="H92" s="4" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="4" t="n"/>
@@ -1439,6 +1540,7 @@
       <c r="E93" s="4" t="n"/>
       <c r="F93" s="4" t="n"/>
       <c r="G93" s="4" t="n"/>
+      <c r="H93" s="4" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="4" t="n"/>
@@ -1448,6 +1550,7 @@
       <c r="E94" s="4" t="n"/>
       <c r="F94" s="4" t="n"/>
       <c r="G94" s="4" t="n"/>
+      <c r="H94" s="4" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="4" t="n"/>
@@ -1457,6 +1560,7 @@
       <c r="E95" s="4" t="n"/>
       <c r="F95" s="4" t="n"/>
       <c r="G95" s="4" t="n"/>
+      <c r="H95" s="4" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="4" t="n"/>
@@ -1466,6 +1570,7 @@
       <c r="E96" s="4" t="n"/>
       <c r="F96" s="4" t="n"/>
       <c r="G96" s="4" t="n"/>
+      <c r="H96" s="4" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="4" t="n"/>
@@ -1475,6 +1580,7 @@
       <c r="E97" s="4" t="n"/>
       <c r="F97" s="4" t="n"/>
       <c r="G97" s="4" t="n"/>
+      <c r="H97" s="4" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="4" t="n"/>
@@ -1484,6 +1590,7 @@
       <c r="E98" s="4" t="n"/>
       <c r="F98" s="4" t="n"/>
       <c r="G98" s="4" t="n"/>
+      <c r="H98" s="4" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="4" t="n"/>
@@ -1493,6 +1600,7 @@
       <c r="E99" s="4" t="n"/>
       <c r="F99" s="4" t="n"/>
       <c r="G99" s="4" t="n"/>
+      <c r="H99" s="4" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="4" t="n"/>
@@ -1502,6 +1610,7 @@
       <c r="E100" s="4" t="n"/>
       <c r="F100" s="4" t="n"/>
       <c r="G100" s="4" t="n"/>
+      <c r="H100" s="4" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="4" t="n"/>
@@ -1511,6 +1620,7 @@
       <c r="E101" s="4" t="n"/>
       <c r="F101" s="4" t="n"/>
       <c r="G101" s="4" t="n"/>
+      <c r="H101" s="4" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="4" t="n"/>
@@ -1520,6 +1630,7 @@
       <c r="E102" s="4" t="n"/>
       <c r="F102" s="4" t="n"/>
       <c r="G102" s="4" t="n"/>
+      <c r="H102" s="4" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="4" t="n"/>
@@ -1529,6 +1640,7 @@
       <c r="E103" s="4" t="n"/>
       <c r="F103" s="4" t="n"/>
       <c r="G103" s="4" t="n"/>
+      <c r="H103" s="4" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="4" t="n"/>
@@ -1538,6 +1650,7 @@
       <c r="E104" s="4" t="n"/>
       <c r="F104" s="4" t="n"/>
       <c r="G104" s="4" t="n"/>
+      <c r="H104" s="4" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="4" t="n"/>
@@ -1547,6 +1660,7 @@
       <c r="E105" s="4" t="n"/>
       <c r="F105" s="4" t="n"/>
       <c r="G105" s="4" t="n"/>
+      <c r="H105" s="4" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="4" t="n"/>
@@ -1556,6 +1670,7 @@
       <c r="E106" s="4" t="n"/>
       <c r="F106" s="4" t="n"/>
       <c r="G106" s="4" t="n"/>
+      <c r="H106" s="4" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="4" t="n"/>
@@ -1565,6 +1680,7 @@
       <c r="E107" s="4" t="n"/>
       <c r="F107" s="4" t="n"/>
       <c r="G107" s="4" t="n"/>
+      <c r="H107" s="4" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="4" t="n"/>
@@ -1574,6 +1690,7 @@
       <c r="E108" s="4" t="n"/>
       <c r="F108" s="4" t="n"/>
       <c r="G108" s="4" t="n"/>
+      <c r="H108" s="4" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="4" t="n"/>
@@ -1583,6 +1700,7 @@
       <c r="E109" s="4" t="n"/>
       <c r="F109" s="4" t="n"/>
       <c r="G109" s="4" t="n"/>
+      <c r="H109" s="4" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="4" t="n"/>
@@ -1592,6 +1710,7 @@
       <c r="E110" s="4" t="n"/>
       <c r="F110" s="4" t="n"/>
       <c r="G110" s="4" t="n"/>
+      <c r="H110" s="4" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="4" t="n"/>
@@ -1601,6 +1720,7 @@
       <c r="E111" s="4" t="n"/>
       <c r="F111" s="4" t="n"/>
       <c r="G111" s="4" t="n"/>
+      <c r="H111" s="4" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="4" t="n"/>
@@ -1610,6 +1730,7 @@
       <c r="E112" s="4" t="n"/>
       <c r="F112" s="4" t="n"/>
       <c r="G112" s="4" t="n"/>
+      <c r="H112" s="4" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="4" t="n"/>
@@ -1619,6 +1740,7 @@
       <c r="E113" s="4" t="n"/>
       <c r="F113" s="4" t="n"/>
       <c r="G113" s="4" t="n"/>
+      <c r="H113" s="4" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="4" t="n"/>
@@ -1628,6 +1750,7 @@
       <c r="E114" s="4" t="n"/>
       <c r="F114" s="4" t="n"/>
       <c r="G114" s="4" t="n"/>
+      <c r="H114" s="4" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="4" t="n"/>
@@ -1637,6 +1760,7 @@
       <c r="E115" s="4" t="n"/>
       <c r="F115" s="4" t="n"/>
       <c r="G115" s="4" t="n"/>
+      <c r="H115" s="4" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="4" t="n"/>
@@ -1646,6 +1770,7 @@
       <c r="E116" s="4" t="n"/>
       <c r="F116" s="4" t="n"/>
       <c r="G116" s="4" t="n"/>
+      <c r="H116" s="4" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="4" t="n"/>
@@ -1655,6 +1780,7 @@
       <c r="E117" s="4" t="n"/>
       <c r="F117" s="4" t="n"/>
       <c r="G117" s="4" t="n"/>
+      <c r="H117" s="4" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="4" t="n"/>
@@ -1664,6 +1790,7 @@
       <c r="E118" s="4" t="n"/>
       <c r="F118" s="4" t="n"/>
       <c r="G118" s="4" t="n"/>
+      <c r="H118" s="4" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="4" t="n"/>
@@ -1673,6 +1800,7 @@
       <c r="E119" s="4" t="n"/>
       <c r="F119" s="4" t="n"/>
       <c r="G119" s="4" t="n"/>
+      <c r="H119" s="4" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="4" t="n"/>
@@ -1682,6 +1810,7 @@
       <c r="E120" s="4" t="n"/>
       <c r="F120" s="4" t="n"/>
       <c r="G120" s="4" t="n"/>
+      <c r="H120" s="4" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="4" t="n"/>
@@ -1691,6 +1820,7 @@
       <c r="E121" s="4" t="n"/>
       <c r="F121" s="4" t="n"/>
       <c r="G121" s="4" t="n"/>
+      <c r="H121" s="4" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="4" t="n"/>
@@ -1700,6 +1830,7 @@
       <c r="E122" s="4" t="n"/>
       <c r="F122" s="4" t="n"/>
       <c r="G122" s="4" t="n"/>
+      <c r="H122" s="4" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="4" t="n"/>
@@ -1709,6 +1840,7 @@
       <c r="E123" s="4" t="n"/>
       <c r="F123" s="4" t="n"/>
       <c r="G123" s="4" t="n"/>
+      <c r="H123" s="4" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="4" t="n"/>
@@ -1718,6 +1850,7 @@
       <c r="E124" s="4" t="n"/>
       <c r="F124" s="4" t="n"/>
       <c r="G124" s="4" t="n"/>
+      <c r="H124" s="4" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="4" t="n"/>
@@ -1727,6 +1860,7 @@
       <c r="E125" s="4" t="n"/>
       <c r="F125" s="4" t="n"/>
       <c r="G125" s="4" t="n"/>
+      <c r="H125" s="4" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="4" t="n"/>
@@ -1736,6 +1870,7 @@
       <c r="E126" s="4" t="n"/>
       <c r="F126" s="4" t="n"/>
       <c r="G126" s="4" t="n"/>
+      <c r="H126" s="4" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="4" t="n"/>
@@ -1745,6 +1880,7 @@
       <c r="E127" s="4" t="n"/>
       <c r="F127" s="4" t="n"/>
       <c r="G127" s="4" t="n"/>
+      <c r="H127" s="4" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="4" t="n"/>
@@ -1754,6 +1890,7 @@
       <c r="E128" s="4" t="n"/>
       <c r="F128" s="4" t="n"/>
       <c r="G128" s="4" t="n"/>
+      <c r="H128" s="4" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="4" t="n"/>
@@ -1763,6 +1900,7 @@
       <c r="E129" s="4" t="n"/>
       <c r="F129" s="4" t="n"/>
       <c r="G129" s="4" t="n"/>
+      <c r="H129" s="4" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="4" t="n"/>
@@ -1772,6 +1910,7 @@
       <c r="E130" s="4" t="n"/>
       <c r="F130" s="4" t="n"/>
       <c r="G130" s="4" t="n"/>
+      <c r="H130" s="4" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="4" t="n"/>
@@ -1781,6 +1920,7 @@
       <c r="E131" s="4" t="n"/>
       <c r="F131" s="4" t="n"/>
       <c r="G131" s="4" t="n"/>
+      <c r="H131" s="4" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="4" t="n"/>
@@ -1790,6 +1930,7 @@
       <c r="E132" s="4" t="n"/>
       <c r="F132" s="4" t="n"/>
       <c r="G132" s="4" t="n"/>
+      <c r="H132" s="4" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="4" t="n"/>
@@ -1799,6 +1940,7 @@
       <c r="E133" s="4" t="n"/>
       <c r="F133" s="4" t="n"/>
       <c r="G133" s="4" t="n"/>
+      <c r="H133" s="4" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="4" t="n"/>
@@ -1808,6 +1950,7 @@
       <c r="E134" s="4" t="n"/>
       <c r="F134" s="4" t="n"/>
       <c r="G134" s="4" t="n"/>
+      <c r="H134" s="4" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="4" t="n"/>
@@ -1817,6 +1960,7 @@
       <c r="E135" s="4" t="n"/>
       <c r="F135" s="4" t="n"/>
       <c r="G135" s="4" t="n"/>
+      <c r="H135" s="4" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="4" t="n"/>
@@ -1826,6 +1970,7 @@
       <c r="E136" s="4" t="n"/>
       <c r="F136" s="4" t="n"/>
       <c r="G136" s="4" t="n"/>
+      <c r="H136" s="4" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="4" t="n"/>
@@ -1835,6 +1980,7 @@
       <c r="E137" s="4" t="n"/>
       <c r="F137" s="4" t="n"/>
       <c r="G137" s="4" t="n"/>
+      <c r="H137" s="4" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="4" t="n"/>
@@ -1844,6 +1990,7 @@
       <c r="E138" s="4" t="n"/>
       <c r="F138" s="4" t="n"/>
       <c r="G138" s="4" t="n"/>
+      <c r="H138" s="4" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="4" t="n"/>
@@ -1853,6 +2000,7 @@
       <c r="E139" s="4" t="n"/>
       <c r="F139" s="4" t="n"/>
       <c r="G139" s="4" t="n"/>
+      <c r="H139" s="4" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="4" t="n"/>
@@ -1862,6 +2010,7 @@
       <c r="E140" s="4" t="n"/>
       <c r="F140" s="4" t="n"/>
       <c r="G140" s="4" t="n"/>
+      <c r="H140" s="4" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="4" t="n"/>
@@ -1871,6 +2020,7 @@
       <c r="E141" s="4" t="n"/>
       <c r="F141" s="4" t="n"/>
       <c r="G141" s="4" t="n"/>
+      <c r="H141" s="4" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="4" t="n"/>
@@ -1880,6 +2030,7 @@
       <c r="E142" s="4" t="n"/>
       <c r="F142" s="4" t="n"/>
       <c r="G142" s="4" t="n"/>
+      <c r="H142" s="4" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="4" t="n"/>
@@ -1889,6 +2040,7 @@
       <c r="E143" s="4" t="n"/>
       <c r="F143" s="4" t="n"/>
       <c r="G143" s="4" t="n"/>
+      <c r="H143" s="4" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="4" t="n"/>
@@ -1898,6 +2050,7 @@
       <c r="E144" s="4" t="n"/>
       <c r="F144" s="4" t="n"/>
       <c r="G144" s="4" t="n"/>
+      <c r="H144" s="4" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="4" t="n"/>
@@ -1907,6 +2060,7 @@
       <c r="E145" s="4" t="n"/>
       <c r="F145" s="4" t="n"/>
       <c r="G145" s="4" t="n"/>
+      <c r="H145" s="4" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="4" t="n"/>
@@ -1916,6 +2070,7 @@
       <c r="E146" s="4" t="n"/>
       <c r="F146" s="4" t="n"/>
       <c r="G146" s="4" t="n"/>
+      <c r="H146" s="4" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="4" t="n"/>
@@ -1925,6 +2080,7 @@
       <c r="E147" s="4" t="n"/>
       <c r="F147" s="4" t="n"/>
       <c r="G147" s="4" t="n"/>
+      <c r="H147" s="4" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="4" t="n"/>
@@ -1934,6 +2090,7 @@
       <c r="E148" s="4" t="n"/>
       <c r="F148" s="4" t="n"/>
       <c r="G148" s="4" t="n"/>
+      <c r="H148" s="4" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="4" t="n"/>
@@ -1943,6 +2100,7 @@
       <c r="E149" s="4" t="n"/>
       <c r="F149" s="4" t="n"/>
       <c r="G149" s="4" t="n"/>
+      <c r="H149" s="4" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="4" t="n"/>
@@ -1952,6 +2110,7 @@
       <c r="E150" s="4" t="n"/>
       <c r="F150" s="4" t="n"/>
       <c r="G150" s="4" t="n"/>
+      <c r="H150" s="4" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="4" t="n"/>
@@ -1961,6 +2120,7 @@
       <c r="E151" s="4" t="n"/>
       <c r="F151" s="4" t="n"/>
       <c r="G151" s="4" t="n"/>
+      <c r="H151" s="4" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="4" t="n"/>
@@ -1970,6 +2130,7 @@
       <c r="E152" s="4" t="n"/>
       <c r="F152" s="4" t="n"/>
       <c r="G152" s="4" t="n"/>
+      <c r="H152" s="4" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="4" t="n"/>
@@ -1979,6 +2140,7 @@
       <c r="E153" s="4" t="n"/>
       <c r="F153" s="4" t="n"/>
       <c r="G153" s="4" t="n"/>
+      <c r="H153" s="4" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="4" t="n"/>
@@ -1988,6 +2150,7 @@
       <c r="E154" s="4" t="n"/>
       <c r="F154" s="4" t="n"/>
       <c r="G154" s="4" t="n"/>
+      <c r="H154" s="4" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="4" t="n"/>
@@ -1997,6 +2160,7 @@
       <c r="E155" s="4" t="n"/>
       <c r="F155" s="4" t="n"/>
       <c r="G155" s="4" t="n"/>
+      <c r="H155" s="4" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="4" t="n"/>
@@ -2006,6 +2170,7 @@
       <c r="E156" s="4" t="n"/>
       <c r="F156" s="4" t="n"/>
       <c r="G156" s="4" t="n"/>
+      <c r="H156" s="4" t="n"/>
     </row>
     <row r="157">
       <c r="A157" s="4" t="n"/>
@@ -2015,6 +2180,7 @@
       <c r="E157" s="4" t="n"/>
       <c r="F157" s="4" t="n"/>
       <c r="G157" s="4" t="n"/>
+      <c r="H157" s="4" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="4" t="n"/>
@@ -2024,6 +2190,7 @@
       <c r="E158" s="4" t="n"/>
       <c r="F158" s="4" t="n"/>
       <c r="G158" s="4" t="n"/>
+      <c r="H158" s="4" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="4" t="n"/>
@@ -2033,6 +2200,7 @@
       <c r="E159" s="4" t="n"/>
       <c r="F159" s="4" t="n"/>
       <c r="G159" s="4" t="n"/>
+      <c r="H159" s="4" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="4" t="n"/>
@@ -2042,6 +2210,7 @@
       <c r="E160" s="4" t="n"/>
       <c r="F160" s="4" t="n"/>
       <c r="G160" s="4" t="n"/>
+      <c r="H160" s="4" t="n"/>
     </row>
     <row r="161">
       <c r="A161" s="4" t="n"/>
@@ -2051,6 +2220,7 @@
       <c r="E161" s="4" t="n"/>
       <c r="F161" s="4" t="n"/>
       <c r="G161" s="4" t="n"/>
+      <c r="H161" s="4" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="4" t="n"/>
@@ -2060,6 +2230,7 @@
       <c r="E162" s="4" t="n"/>
       <c r="F162" s="4" t="n"/>
       <c r="G162" s="4" t="n"/>
+      <c r="H162" s="4" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="4" t="n"/>
@@ -2069,6 +2240,7 @@
       <c r="E163" s="4" t="n"/>
       <c r="F163" s="4" t="n"/>
       <c r="G163" s="4" t="n"/>
+      <c r="H163" s="4" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="4" t="n"/>
@@ -2078,6 +2250,7 @@
       <c r="E164" s="4" t="n"/>
       <c r="F164" s="4" t="n"/>
       <c r="G164" s="4" t="n"/>
+      <c r="H164" s="4" t="n"/>
     </row>
     <row r="165">
       <c r="A165" s="4" t="n"/>
@@ -2087,6 +2260,7 @@
       <c r="E165" s="4" t="n"/>
       <c r="F165" s="4" t="n"/>
       <c r="G165" s="4" t="n"/>
+      <c r="H165" s="4" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="4" t="n"/>
@@ -2096,6 +2270,7 @@
       <c r="E166" s="4" t="n"/>
       <c r="F166" s="4" t="n"/>
       <c r="G166" s="4" t="n"/>
+      <c r="H166" s="4" t="n"/>
     </row>
     <row r="167">
       <c r="A167" s="4" t="n"/>
@@ -2105,6 +2280,7 @@
       <c r="E167" s="4" t="n"/>
       <c r="F167" s="4" t="n"/>
       <c r="G167" s="4" t="n"/>
+      <c r="H167" s="4" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="4" t="n"/>
@@ -2114,6 +2290,7 @@
       <c r="E168" s="4" t="n"/>
       <c r="F168" s="4" t="n"/>
       <c r="G168" s="4" t="n"/>
+      <c r="H168" s="4" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="4" t="n"/>
@@ -2123,6 +2300,7 @@
       <c r="E169" s="4" t="n"/>
       <c r="F169" s="4" t="n"/>
       <c r="G169" s="4" t="n"/>
+      <c r="H169" s="4" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="4" t="n"/>
@@ -2132,6 +2310,7 @@
       <c r="E170" s="4" t="n"/>
       <c r="F170" s="4" t="n"/>
       <c r="G170" s="4" t="n"/>
+      <c r="H170" s="4" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="4" t="n"/>
@@ -2141,6 +2320,7 @@
       <c r="E171" s="4" t="n"/>
       <c r="F171" s="4" t="n"/>
       <c r="G171" s="4" t="n"/>
+      <c r="H171" s="4" t="n"/>
     </row>
     <row r="172">
       <c r="A172" s="4" t="n"/>
@@ -2150,6 +2330,7 @@
       <c r="E172" s="4" t="n"/>
       <c r="F172" s="4" t="n"/>
       <c r="G172" s="4" t="n"/>
+      <c r="H172" s="4" t="n"/>
     </row>
     <row r="173">
       <c r="A173" s="4" t="n"/>
@@ -2159,6 +2340,7 @@
       <c r="E173" s="4" t="n"/>
       <c r="F173" s="4" t="n"/>
       <c r="G173" s="4" t="n"/>
+      <c r="H173" s="4" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="4" t="n"/>
@@ -2168,6 +2350,7 @@
       <c r="E174" s="4" t="n"/>
       <c r="F174" s="4" t="n"/>
       <c r="G174" s="4" t="n"/>
+      <c r="H174" s="4" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="4" t="n"/>
@@ -2177,6 +2360,7 @@
       <c r="E175" s="4" t="n"/>
       <c r="F175" s="4" t="n"/>
       <c r="G175" s="4" t="n"/>
+      <c r="H175" s="4" t="n"/>
     </row>
     <row r="176">
       <c r="A176" s="4" t="n"/>
@@ -2186,6 +2370,7 @@
       <c r="E176" s="4" t="n"/>
       <c r="F176" s="4" t="n"/>
       <c r="G176" s="4" t="n"/>
+      <c r="H176" s="4" t="n"/>
     </row>
     <row r="177">
       <c r="A177" s="4" t="n"/>
@@ -2195,6 +2380,7 @@
       <c r="E177" s="4" t="n"/>
       <c r="F177" s="4" t="n"/>
       <c r="G177" s="4" t="n"/>
+      <c r="H177" s="4" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="4" t="n"/>
@@ -2204,6 +2390,7 @@
       <c r="E178" s="4" t="n"/>
       <c r="F178" s="4" t="n"/>
       <c r="G178" s="4" t="n"/>
+      <c r="H178" s="4" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="4" t="n"/>
@@ -2213,6 +2400,7 @@
       <c r="E179" s="4" t="n"/>
       <c r="F179" s="4" t="n"/>
       <c r="G179" s="4" t="n"/>
+      <c r="H179" s="4" t="n"/>
     </row>
     <row r="180">
       <c r="A180" s="4" t="n"/>
@@ -2222,6 +2410,7 @@
       <c r="E180" s="4" t="n"/>
       <c r="F180" s="4" t="n"/>
       <c r="G180" s="4" t="n"/>
+      <c r="H180" s="4" t="n"/>
     </row>
     <row r="181">
       <c r="A181" s="4" t="n"/>
@@ -2231,6 +2420,7 @@
       <c r="E181" s="4" t="n"/>
       <c r="F181" s="4" t="n"/>
       <c r="G181" s="4" t="n"/>
+      <c r="H181" s="4" t="n"/>
     </row>
     <row r="182">
       <c r="A182" s="4" t="n"/>
@@ -2240,6 +2430,7 @@
       <c r="E182" s="4" t="n"/>
       <c r="F182" s="4" t="n"/>
       <c r="G182" s="4" t="n"/>
+      <c r="H182" s="4" t="n"/>
     </row>
     <row r="183">
       <c r="A183" s="4" t="n"/>
@@ -2249,6 +2440,7 @@
       <c r="E183" s="4" t="n"/>
       <c r="F183" s="4" t="n"/>
       <c r="G183" s="4" t="n"/>
+      <c r="H183" s="4" t="n"/>
     </row>
     <row r="184">
       <c r="A184" s="4" t="n"/>
@@ -2258,6 +2450,7 @@
       <c r="E184" s="4" t="n"/>
       <c r="F184" s="4" t="n"/>
       <c r="G184" s="4" t="n"/>
+      <c r="H184" s="4" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="4" t="n"/>
@@ -2267,6 +2460,7 @@
       <c r="E185" s="4" t="n"/>
       <c r="F185" s="4" t="n"/>
       <c r="G185" s="4" t="n"/>
+      <c r="H185" s="4" t="n"/>
     </row>
     <row r="186">
       <c r="A186" s="4" t="n"/>
@@ -2276,6 +2470,7 @@
       <c r="E186" s="4" t="n"/>
       <c r="F186" s="4" t="n"/>
       <c r="G186" s="4" t="n"/>
+      <c r="H186" s="4" t="n"/>
     </row>
     <row r="187">
       <c r="A187" s="4" t="n"/>
@@ -2285,6 +2480,7 @@
       <c r="E187" s="4" t="n"/>
       <c r="F187" s="4" t="n"/>
       <c r="G187" s="4" t="n"/>
+      <c r="H187" s="4" t="n"/>
     </row>
     <row r="188">
       <c r="A188" s="4" t="n"/>
@@ -2294,6 +2490,7 @@
       <c r="E188" s="4" t="n"/>
       <c r="F188" s="4" t="n"/>
       <c r="G188" s="4" t="n"/>
+      <c r="H188" s="4" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="4" t="n"/>
@@ -2303,6 +2500,7 @@
       <c r="E189" s="4" t="n"/>
       <c r="F189" s="4" t="n"/>
       <c r="G189" s="4" t="n"/>
+      <c r="H189" s="4" t="n"/>
     </row>
     <row r="190">
       <c r="A190" s="4" t="n"/>
@@ -2312,6 +2510,7 @@
       <c r="E190" s="4" t="n"/>
       <c r="F190" s="4" t="n"/>
       <c r="G190" s="4" t="n"/>
+      <c r="H190" s="4" t="n"/>
     </row>
     <row r="191">
       <c r="A191" s="4" t="n"/>
@@ -2321,6 +2520,7 @@
       <c r="E191" s="4" t="n"/>
       <c r="F191" s="4" t="n"/>
       <c r="G191" s="4" t="n"/>
+      <c r="H191" s="4" t="n"/>
     </row>
     <row r="192">
       <c r="A192" s="4" t="n"/>
@@ -2330,6 +2530,7 @@
       <c r="E192" s="4" t="n"/>
       <c r="F192" s="4" t="n"/>
       <c r="G192" s="4" t="n"/>
+      <c r="H192" s="4" t="n"/>
     </row>
     <row r="193">
       <c r="A193" s="4" t="n"/>
@@ -2339,6 +2540,7 @@
       <c r="E193" s="4" t="n"/>
       <c r="F193" s="4" t="n"/>
       <c r="G193" s="4" t="n"/>
+      <c r="H193" s="4" t="n"/>
     </row>
     <row r="194">
       <c r="A194" s="4" t="n"/>
@@ -2348,6 +2550,7 @@
       <c r="E194" s="4" t="n"/>
       <c r="F194" s="4" t="n"/>
       <c r="G194" s="4" t="n"/>
+      <c r="H194" s="4" t="n"/>
     </row>
     <row r="195">
       <c r="A195" s="4" t="n"/>
@@ -2357,6 +2560,7 @@
       <c r="E195" s="4" t="n"/>
       <c r="F195" s="4" t="n"/>
       <c r="G195" s="4" t="n"/>
+      <c r="H195" s="4" t="n"/>
     </row>
     <row r="196">
       <c r="A196" s="4" t="n"/>
@@ -2366,6 +2570,7 @@
       <c r="E196" s="4" t="n"/>
       <c r="F196" s="4" t="n"/>
       <c r="G196" s="4" t="n"/>
+      <c r="H196" s="4" t="n"/>
     </row>
     <row r="197">
       <c r="A197" s="4" t="n"/>
@@ -2375,6 +2580,7 @@
       <c r="E197" s="4" t="n"/>
       <c r="F197" s="4" t="n"/>
       <c r="G197" s="4" t="n"/>
+      <c r="H197" s="4" t="n"/>
     </row>
     <row r="198">
       <c r="A198" s="4" t="n"/>
@@ -2384,6 +2590,7 @@
       <c r="E198" s="4" t="n"/>
       <c r="F198" s="4" t="n"/>
       <c r="G198" s="4" t="n"/>
+      <c r="H198" s="4" t="n"/>
     </row>
     <row r="199">
       <c r="A199" s="4" t="n"/>
@@ -2393,6 +2600,7 @@
       <c r="E199" s="4" t="n"/>
       <c r="F199" s="4" t="n"/>
       <c r="G199" s="4" t="n"/>
+      <c r="H199" s="4" t="n"/>
     </row>
     <row r="200">
       <c r="A200" s="4" t="n"/>
@@ -2402,6 +2610,7 @@
       <c r="E200" s="4" t="n"/>
       <c r="F200" s="4" t="n"/>
       <c r="G200" s="4" t="n"/>
+      <c r="H200" s="4" t="n"/>
     </row>
     <row r="201">
       <c r="A201" s="4" t="n"/>
@@ -2411,6 +2620,7 @@
       <c r="E201" s="4" t="n"/>
       <c r="F201" s="4" t="n"/>
       <c r="G201" s="4" t="n"/>
+      <c r="H201" s="4" t="n"/>
     </row>
     <row r="202">
       <c r="A202" s="4" t="n"/>
@@ -2420,6 +2630,7 @@
       <c r="E202" s="4" t="n"/>
       <c r="F202" s="4" t="n"/>
       <c r="G202" s="4" t="n"/>
+      <c r="H202" s="4" t="n"/>
     </row>
     <row r="203">
       <c r="A203" s="4" t="n"/>
@@ -2429,6 +2640,7 @@
       <c r="E203" s="4" t="n"/>
       <c r="F203" s="4" t="n"/>
       <c r="G203" s="4" t="n"/>
+      <c r="H203" s="4" t="n"/>
     </row>
     <row r="204">
       <c r="A204" s="4" t="n"/>
@@ -2438,6 +2650,7 @@
       <c r="E204" s="4" t="n"/>
       <c r="F204" s="4" t="n"/>
       <c r="G204" s="4" t="n"/>
+      <c r="H204" s="4" t="n"/>
     </row>
     <row r="205">
       <c r="A205" s="4" t="n"/>
@@ -2447,6 +2660,7 @@
       <c r="E205" s="4" t="n"/>
       <c r="F205" s="4" t="n"/>
       <c r="G205" s="4" t="n"/>
+      <c r="H205" s="4" t="n"/>
     </row>
     <row r="206">
       <c r="A206" s="4" t="n"/>
@@ -2456,6 +2670,7 @@
       <c r="E206" s="4" t="n"/>
       <c r="F206" s="4" t="n"/>
       <c r="G206" s="4" t="n"/>
+      <c r="H206" s="4" t="n"/>
     </row>
     <row r="207">
       <c r="A207" s="4" t="n"/>
@@ -2465,6 +2680,7 @@
       <c r="E207" s="4" t="n"/>
       <c r="F207" s="4" t="n"/>
       <c r="G207" s="4" t="n"/>
+      <c r="H207" s="4" t="n"/>
     </row>
     <row r="208">
       <c r="A208" s="4" t="n"/>
@@ -2474,6 +2690,7 @@
       <c r="E208" s="4" t="n"/>
       <c r="F208" s="4" t="n"/>
       <c r="G208" s="4" t="n"/>
+      <c r="H208" s="4" t="n"/>
     </row>
     <row r="209">
       <c r="A209" s="4" t="n"/>
@@ -2483,6 +2700,7 @@
       <c r="E209" s="4" t="n"/>
       <c r="F209" s="4" t="n"/>
       <c r="G209" s="4" t="n"/>
+      <c r="H209" s="4" t="n"/>
     </row>
     <row r="210">
       <c r="A210" s="4" t="n"/>
@@ -2492,6 +2710,7 @@
       <c r="E210" s="4" t="n"/>
       <c r="F210" s="4" t="n"/>
       <c r="G210" s="4" t="n"/>
+      <c r="H210" s="4" t="n"/>
     </row>
     <row r="211">
       <c r="A211" s="4" t="n"/>
@@ -2501,6 +2720,7 @@
       <c r="E211" s="4" t="n"/>
       <c r="F211" s="4" t="n"/>
       <c r="G211" s="4" t="n"/>
+      <c r="H211" s="4" t="n"/>
     </row>
     <row r="212">
       <c r="A212" s="4" t="n"/>
@@ -2510,6 +2730,7 @@
       <c r="E212" s="4" t="n"/>
       <c r="F212" s="4" t="n"/>
       <c r="G212" s="4" t="n"/>
+      <c r="H212" s="4" t="n"/>
     </row>
     <row r="213">
       <c r="A213" s="4" t="n"/>
@@ -2519,6 +2740,7 @@
       <c r="E213" s="4" t="n"/>
       <c r="F213" s="4" t="n"/>
       <c r="G213" s="4" t="n"/>
+      <c r="H213" s="4" t="n"/>
     </row>
     <row r="214">
       <c r="A214" s="4" t="n"/>
@@ -2528,6 +2750,7 @@
       <c r="E214" s="4" t="n"/>
       <c r="F214" s="4" t="n"/>
       <c r="G214" s="4" t="n"/>
+      <c r="H214" s="4" t="n"/>
     </row>
     <row r="215">
       <c r="A215" s="4" t="n"/>
@@ -2537,6 +2760,7 @@
       <c r="E215" s="4" t="n"/>
       <c r="F215" s="4" t="n"/>
       <c r="G215" s="4" t="n"/>
+      <c r="H215" s="4" t="n"/>
     </row>
     <row r="216">
       <c r="A216" s="4" t="n"/>
@@ -2546,6 +2770,7 @@
       <c r="E216" s="4" t="n"/>
       <c r="F216" s="4" t="n"/>
       <c r="G216" s="4" t="n"/>
+      <c r="H216" s="4" t="n"/>
     </row>
     <row r="217">
       <c r="A217" s="4" t="n"/>
@@ -2555,6 +2780,7 @@
       <c r="E217" s="4" t="n"/>
       <c r="F217" s="4" t="n"/>
       <c r="G217" s="4" t="n"/>
+      <c r="H217" s="4" t="n"/>
     </row>
     <row r="218">
       <c r="A218" s="4" t="n"/>
@@ -2564,6 +2790,7 @@
       <c r="E218" s="4" t="n"/>
       <c r="F218" s="4" t="n"/>
       <c r="G218" s="4" t="n"/>
+      <c r="H218" s="4" t="n"/>
     </row>
     <row r="219">
       <c r="A219" s="4" t="n"/>
@@ -2573,6 +2800,7 @@
       <c r="E219" s="4" t="n"/>
       <c r="F219" s="4" t="n"/>
       <c r="G219" s="4" t="n"/>
+      <c r="H219" s="4" t="n"/>
     </row>
     <row r="220">
       <c r="A220" s="4" t="n"/>
@@ -2582,6 +2810,7 @@
       <c r="E220" s="4" t="n"/>
       <c r="F220" s="4" t="n"/>
       <c r="G220" s="4" t="n"/>
+      <c r="H220" s="4" t="n"/>
     </row>
     <row r="221">
       <c r="A221" s="4" t="n"/>
@@ -2591,6 +2820,7 @@
       <c r="E221" s="4" t="n"/>
       <c r="F221" s="4" t="n"/>
       <c r="G221" s="4" t="n"/>
+      <c r="H221" s="4" t="n"/>
     </row>
     <row r="222">
       <c r="A222" s="4" t="n"/>
@@ -2600,6 +2830,7 @@
       <c r="E222" s="4" t="n"/>
       <c r="F222" s="4" t="n"/>
       <c r="G222" s="4" t="n"/>
+      <c r="H222" s="4" t="n"/>
     </row>
     <row r="223">
       <c r="A223" s="4" t="n"/>
@@ -2609,6 +2840,7 @@
       <c r="E223" s="4" t="n"/>
       <c r="F223" s="4" t="n"/>
       <c r="G223" s="4" t="n"/>
+      <c r="H223" s="4" t="n"/>
     </row>
     <row r="224">
       <c r="A224" s="4" t="n"/>
@@ -2618,6 +2850,7 @@
       <c r="E224" s="4" t="n"/>
       <c r="F224" s="4" t="n"/>
       <c r="G224" s="4" t="n"/>
+      <c r="H224" s="4" t="n"/>
     </row>
     <row r="225">
       <c r="A225" s="4" t="n"/>
@@ -2627,6 +2860,7 @@
       <c r="E225" s="4" t="n"/>
       <c r="F225" s="4" t="n"/>
       <c r="G225" s="4" t="n"/>
+      <c r="H225" s="4" t="n"/>
     </row>
     <row r="226">
       <c r="A226" s="4" t="n"/>
@@ -2636,6 +2870,7 @@
       <c r="E226" s="4" t="n"/>
       <c r="F226" s="4" t="n"/>
       <c r="G226" s="4" t="n"/>
+      <c r="H226" s="4" t="n"/>
     </row>
     <row r="227">
       <c r="A227" s="4" t="n"/>
@@ -2645,6 +2880,7 @@
       <c r="E227" s="4" t="n"/>
       <c r="F227" s="4" t="n"/>
       <c r="G227" s="4" t="n"/>
+      <c r="H227" s="4" t="n"/>
     </row>
     <row r="228">
       <c r="A228" s="4" t="n"/>
@@ -2654,6 +2890,7 @@
       <c r="E228" s="4" t="n"/>
       <c r="F228" s="4" t="n"/>
       <c r="G228" s="4" t="n"/>
+      <c r="H228" s="4" t="n"/>
     </row>
     <row r="229">
       <c r="A229" s="4" t="n"/>
@@ -2663,6 +2900,7 @@
       <c r="E229" s="4" t="n"/>
       <c r="F229" s="4" t="n"/>
       <c r="G229" s="4" t="n"/>
+      <c r="H229" s="4" t="n"/>
     </row>
     <row r="230">
       <c r="A230" s="4" t="n"/>
@@ -2672,6 +2910,7 @@
       <c r="E230" s="4" t="n"/>
       <c r="F230" s="4" t="n"/>
       <c r="G230" s="4" t="n"/>
+      <c r="H230" s="4" t="n"/>
     </row>
     <row r="231">
       <c r="A231" s="4" t="n"/>
@@ -2681,6 +2920,7 @@
       <c r="E231" s="4" t="n"/>
       <c r="F231" s="4" t="n"/>
       <c r="G231" s="4" t="n"/>
+      <c r="H231" s="4" t="n"/>
     </row>
     <row r="232">
       <c r="A232" s="4" t="n"/>
@@ -2690,6 +2930,7 @@
       <c r="E232" s="4" t="n"/>
       <c r="F232" s="4" t="n"/>
       <c r="G232" s="4" t="n"/>
+      <c r="H232" s="4" t="n"/>
     </row>
     <row r="233">
       <c r="A233" s="4" t="n"/>
@@ -2699,6 +2940,7 @@
       <c r="E233" s="4" t="n"/>
       <c r="F233" s="4" t="n"/>
       <c r="G233" s="4" t="n"/>
+      <c r="H233" s="4" t="n"/>
     </row>
     <row r="234">
       <c r="A234" s="4" t="n"/>
@@ -2708,6 +2950,7 @@
       <c r="E234" s="4" t="n"/>
       <c r="F234" s="4" t="n"/>
       <c r="G234" s="4" t="n"/>
+      <c r="H234" s="4" t="n"/>
     </row>
     <row r="235">
       <c r="A235" s="4" t="n"/>
@@ -2717,6 +2960,7 @@
       <c r="E235" s="4" t="n"/>
       <c r="F235" s="4" t="n"/>
       <c r="G235" s="4" t="n"/>
+      <c r="H235" s="4" t="n"/>
     </row>
     <row r="236">
       <c r="A236" s="4" t="n"/>
@@ -2726,6 +2970,7 @@
       <c r="E236" s="4" t="n"/>
       <c r="F236" s="4" t="n"/>
       <c r="G236" s="4" t="n"/>
+      <c r="H236" s="4" t="n"/>
     </row>
     <row r="237">
       <c r="A237" s="4" t="n"/>
@@ -2735,6 +2980,7 @@
       <c r="E237" s="4" t="n"/>
       <c r="F237" s="4" t="n"/>
       <c r="G237" s="4" t="n"/>
+      <c r="H237" s="4" t="n"/>
     </row>
     <row r="238">
       <c r="A238" s="4" t="n"/>
@@ -2744,6 +2990,7 @@
       <c r="E238" s="4" t="n"/>
       <c r="F238" s="4" t="n"/>
       <c r="G238" s="4" t="n"/>
+      <c r="H238" s="4" t="n"/>
     </row>
     <row r="239">
       <c r="A239" s="4" t="n"/>
@@ -2753,6 +3000,7 @@
       <c r="E239" s="4" t="n"/>
       <c r="F239" s="4" t="n"/>
       <c r="G239" s="4" t="n"/>
+      <c r="H239" s="4" t="n"/>
     </row>
     <row r="240">
       <c r="A240" s="4" t="n"/>
@@ -2762,6 +3010,7 @@
       <c r="E240" s="4" t="n"/>
       <c r="F240" s="4" t="n"/>
       <c r="G240" s="4" t="n"/>
+      <c r="H240" s="4" t="n"/>
     </row>
     <row r="241">
       <c r="A241" s="4" t="n"/>
@@ -2771,6 +3020,7 @@
       <c r="E241" s="4" t="n"/>
       <c r="F241" s="4" t="n"/>
       <c r="G241" s="4" t="n"/>
+      <c r="H241" s="4" t="n"/>
     </row>
     <row r="242">
       <c r="A242" s="4" t="n"/>
@@ -2780,6 +3030,7 @@
       <c r="E242" s="4" t="n"/>
       <c r="F242" s="4" t="n"/>
       <c r="G242" s="4" t="n"/>
+      <c r="H242" s="4" t="n"/>
     </row>
     <row r="243">
       <c r="A243" s="4" t="n"/>
@@ -2789,6 +3040,7 @@
       <c r="E243" s="4" t="n"/>
       <c r="F243" s="4" t="n"/>
       <c r="G243" s="4" t="n"/>
+      <c r="H243" s="4" t="n"/>
     </row>
     <row r="244">
       <c r="A244" s="4" t="n"/>
@@ -2798,6 +3050,7 @@
       <c r="E244" s="4" t="n"/>
       <c r="F244" s="4" t="n"/>
       <c r="G244" s="4" t="n"/>
+      <c r="H244" s="4" t="n"/>
     </row>
     <row r="245">
       <c r="A245" s="4" t="n"/>
@@ -2807,6 +3060,7 @@
       <c r="E245" s="4" t="n"/>
       <c r="F245" s="4" t="n"/>
       <c r="G245" s="4" t="n"/>
+      <c r="H245" s="4" t="n"/>
     </row>
     <row r="246">
       <c r="A246" s="4" t="n"/>
@@ -2816,6 +3070,7 @@
       <c r="E246" s="4" t="n"/>
       <c r="F246" s="4" t="n"/>
       <c r="G246" s="4" t="n"/>
+      <c r="H246" s="4" t="n"/>
     </row>
     <row r="247">
       <c r="A247" s="4" t="n"/>
@@ -2825,6 +3080,7 @@
       <c r="E247" s="4" t="n"/>
       <c r="F247" s="4" t="n"/>
       <c r="G247" s="4" t="n"/>
+      <c r="H247" s="4" t="n"/>
     </row>
     <row r="248">
       <c r="A248" s="4" t="n"/>
@@ -2834,6 +3090,7 @@
       <c r="E248" s="4" t="n"/>
       <c r="F248" s="4" t="n"/>
       <c r="G248" s="4" t="n"/>
+      <c r="H248" s="4" t="n"/>
     </row>
     <row r="249">
       <c r="A249" s="4" t="n"/>
@@ -2843,6 +3100,7 @@
       <c r="E249" s="4" t="n"/>
       <c r="F249" s="4" t="n"/>
       <c r="G249" s="4" t="n"/>
+      <c r="H249" s="4" t="n"/>
     </row>
     <row r="250">
       <c r="A250" s="4" t="n"/>
@@ -2852,6 +3110,7 @@
       <c r="E250" s="4" t="n"/>
       <c r="F250" s="4" t="n"/>
       <c r="G250" s="4" t="n"/>
+      <c r="H250" s="4" t="n"/>
     </row>
     <row r="251">
       <c r="A251" s="4" t="n"/>
@@ -2861,6 +3120,7 @@
       <c r="E251" s="4" t="n"/>
       <c r="F251" s="4" t="n"/>
       <c r="G251" s="4" t="n"/>
+      <c r="H251" s="4" t="n"/>
     </row>
     <row r="252">
       <c r="A252" s="4" t="n"/>
@@ -2870,6 +3130,7 @@
       <c r="E252" s="4" t="n"/>
       <c r="F252" s="4" t="n"/>
       <c r="G252" s="4" t="n"/>
+      <c r="H252" s="4" t="n"/>
     </row>
     <row r="253">
       <c r="A253" s="4" t="n"/>
@@ -2879,6 +3140,7 @@
       <c r="E253" s="4" t="n"/>
       <c r="F253" s="4" t="n"/>
       <c r="G253" s="4" t="n"/>
+      <c r="H253" s="4" t="n"/>
     </row>
     <row r="254">
       <c r="A254" s="4" t="n"/>
@@ -2888,6 +3150,7 @@
       <c r="E254" s="4" t="n"/>
       <c r="F254" s="4" t="n"/>
       <c r="G254" s="4" t="n"/>
+      <c r="H254" s="4" t="n"/>
     </row>
     <row r="255">
       <c r="A255" s="4" t="n"/>
@@ -2897,6 +3160,7 @@
       <c r="E255" s="4" t="n"/>
       <c r="F255" s="4" t="n"/>
       <c r="G255" s="4" t="n"/>
+      <c r="H255" s="4" t="n"/>
     </row>
     <row r="256">
       <c r="A256" s="4" t="n"/>
@@ -2906,6 +3170,7 @@
       <c r="E256" s="4" t="n"/>
       <c r="F256" s="4" t="n"/>
       <c r="G256" s="4" t="n"/>
+      <c r="H256" s="4" t="n"/>
     </row>
     <row r="257">
       <c r="A257" s="4" t="n"/>
@@ -2915,6 +3180,7 @@
       <c r="E257" s="4" t="n"/>
       <c r="F257" s="4" t="n"/>
       <c r="G257" s="4" t="n"/>
+      <c r="H257" s="4" t="n"/>
     </row>
     <row r="258">
       <c r="A258" s="4" t="n"/>
@@ -2924,6 +3190,7 @@
       <c r="E258" s="4" t="n"/>
       <c r="F258" s="4" t="n"/>
       <c r="G258" s="4" t="n"/>
+      <c r="H258" s="4" t="n"/>
     </row>
     <row r="259">
       <c r="A259" s="4" t="n"/>
@@ -2933,6 +3200,7 @@
       <c r="E259" s="4" t="n"/>
       <c r="F259" s="4" t="n"/>
       <c r="G259" s="4" t="n"/>
+      <c r="H259" s="4" t="n"/>
     </row>
     <row r="260">
       <c r="A260" s="4" t="n"/>
@@ -2942,6 +3210,7 @@
       <c r="E260" s="4" t="n"/>
       <c r="F260" s="4" t="n"/>
       <c r="G260" s="4" t="n"/>
+      <c r="H260" s="4" t="n"/>
     </row>
     <row r="261">
       <c r="A261" s="4" t="n"/>
@@ -2951,6 +3220,7 @@
       <c r="E261" s="4" t="n"/>
       <c r="F261" s="4" t="n"/>
       <c r="G261" s="4" t="n"/>
+      <c r="H261" s="4" t="n"/>
     </row>
     <row r="262">
       <c r="A262" s="4" t="n"/>
@@ -2960,6 +3230,7 @@
       <c r="E262" s="4" t="n"/>
       <c r="F262" s="4" t="n"/>
       <c r="G262" s="4" t="n"/>
+      <c r="H262" s="4" t="n"/>
     </row>
     <row r="263">
       <c r="A263" s="4" t="n"/>
@@ -2969,6 +3240,7 @@
       <c r="E263" s="4" t="n"/>
       <c r="F263" s="4" t="n"/>
       <c r="G263" s="4" t="n"/>
+      <c r="H263" s="4" t="n"/>
     </row>
     <row r="264">
       <c r="A264" s="4" t="n"/>
@@ -2978,6 +3250,7 @@
       <c r="E264" s="4" t="n"/>
       <c r="F264" s="4" t="n"/>
       <c r="G264" s="4" t="n"/>
+      <c r="H264" s="4" t="n"/>
     </row>
     <row r="265">
       <c r="A265" s="4" t="n"/>
@@ -2987,6 +3260,7 @@
       <c r="E265" s="4" t="n"/>
       <c r="F265" s="4" t="n"/>
       <c r="G265" s="4" t="n"/>
+      <c r="H265" s="4" t="n"/>
     </row>
     <row r="266">
       <c r="A266" s="4" t="n"/>
@@ -2996,6 +3270,7 @@
       <c r="E266" s="4" t="n"/>
       <c r="F266" s="4" t="n"/>
       <c r="G266" s="4" t="n"/>
+      <c r="H266" s="4" t="n"/>
     </row>
     <row r="267">
       <c r="A267" s="4" t="n"/>
@@ -3005,6 +3280,7 @@
       <c r="E267" s="4" t="n"/>
       <c r="F267" s="4" t="n"/>
       <c r="G267" s="4" t="n"/>
+      <c r="H267" s="4" t="n"/>
     </row>
     <row r="268">
       <c r="A268" s="4" t="n"/>
@@ -3014,6 +3290,7 @@
       <c r="E268" s="4" t="n"/>
       <c r="F268" s="4" t="n"/>
       <c r="G268" s="4" t="n"/>
+      <c r="H268" s="4" t="n"/>
     </row>
     <row r="269">
       <c r="A269" s="4" t="n"/>
@@ -3023,6 +3300,7 @@
       <c r="E269" s="4" t="n"/>
       <c r="F269" s="4" t="n"/>
       <c r="G269" s="4" t="n"/>
+      <c r="H269" s="4" t="n"/>
     </row>
     <row r="270">
       <c r="A270" s="4" t="n"/>
@@ -3032,6 +3310,7 @@
       <c r="E270" s="4" t="n"/>
       <c r="F270" s="4" t="n"/>
       <c r="G270" s="4" t="n"/>
+      <c r="H270" s="4" t="n"/>
     </row>
     <row r="271">
       <c r="A271" s="4" t="n"/>
@@ -3041,6 +3320,7 @@
       <c r="E271" s="4" t="n"/>
       <c r="F271" s="4" t="n"/>
       <c r="G271" s="4" t="n"/>
+      <c r="H271" s="4" t="n"/>
     </row>
     <row r="272">
       <c r="A272" s="4" t="n"/>
@@ -3050,6 +3330,7 @@
       <c r="E272" s="4" t="n"/>
       <c r="F272" s="4" t="n"/>
       <c r="G272" s="4" t="n"/>
+      <c r="H272" s="4" t="n"/>
     </row>
     <row r="273">
       <c r="A273" s="4" t="n"/>
@@ -3059,6 +3340,7 @@
       <c r="E273" s="4" t="n"/>
       <c r="F273" s="4" t="n"/>
       <c r="G273" s="4" t="n"/>
+      <c r="H273" s="4" t="n"/>
     </row>
     <row r="274">
       <c r="A274" s="4" t="n"/>
@@ -3068,6 +3350,7 @@
       <c r="E274" s="4" t="n"/>
       <c r="F274" s="4" t="n"/>
       <c r="G274" s="4" t="n"/>
+      <c r="H274" s="4" t="n"/>
     </row>
     <row r="275">
       <c r="A275" s="4" t="n"/>
@@ -3077,6 +3360,7 @@
       <c r="E275" s="4" t="n"/>
       <c r="F275" s="4" t="n"/>
       <c r="G275" s="4" t="n"/>
+      <c r="H275" s="4" t="n"/>
     </row>
     <row r="276">
       <c r="A276" s="4" t="n"/>
@@ -3086,6 +3370,7 @@
       <c r="E276" s="4" t="n"/>
       <c r="F276" s="4" t="n"/>
       <c r="G276" s="4" t="n"/>
+      <c r="H276" s="4" t="n"/>
     </row>
     <row r="277">
       <c r="A277" s="4" t="n"/>
@@ -3095,6 +3380,7 @@
       <c r="E277" s="4" t="n"/>
       <c r="F277" s="4" t="n"/>
       <c r="G277" s="4" t="n"/>
+      <c r="H277" s="4" t="n"/>
     </row>
     <row r="278">
       <c r="A278" s="4" t="n"/>
@@ -3104,6 +3390,7 @@
       <c r="E278" s="4" t="n"/>
       <c r="F278" s="4" t="n"/>
       <c r="G278" s="4" t="n"/>
+      <c r="H278" s="4" t="n"/>
     </row>
     <row r="279">
       <c r="A279" s="4" t="n"/>
@@ -3113,6 +3400,7 @@
       <c r="E279" s="4" t="n"/>
       <c r="F279" s="4" t="n"/>
       <c r="G279" s="4" t="n"/>
+      <c r="H279" s="4" t="n"/>
     </row>
     <row r="280">
       <c r="A280" s="4" t="n"/>
@@ -3122,6 +3410,7 @@
       <c r="E280" s="4" t="n"/>
       <c r="F280" s="4" t="n"/>
       <c r="G280" s="4" t="n"/>
+      <c r="H280" s="4" t="n"/>
     </row>
     <row r="281">
       <c r="A281" s="4" t="n"/>
@@ -3131,6 +3420,7 @@
       <c r="E281" s="4" t="n"/>
       <c r="F281" s="4" t="n"/>
       <c r="G281" s="4" t="n"/>
+      <c r="H281" s="4" t="n"/>
     </row>
     <row r="282">
       <c r="A282" s="4" t="n"/>
@@ -3140,6 +3430,7 @@
       <c r="E282" s="4" t="n"/>
       <c r="F282" s="4" t="n"/>
       <c r="G282" s="4" t="n"/>
+      <c r="H282" s="4" t="n"/>
     </row>
     <row r="283">
       <c r="A283" s="4" t="n"/>
@@ -3149,6 +3440,7 @@
       <c r="E283" s="4" t="n"/>
       <c r="F283" s="4" t="n"/>
       <c r="G283" s="4" t="n"/>
+      <c r="H283" s="4" t="n"/>
     </row>
     <row r="284">
       <c r="A284" s="4" t="n"/>
@@ -3158,6 +3450,7 @@
       <c r="E284" s="4" t="n"/>
       <c r="F284" s="4" t="n"/>
       <c r="G284" s="4" t="n"/>
+      <c r="H284" s="4" t="n"/>
     </row>
     <row r="285">
       <c r="A285" s="4" t="n"/>
@@ -3167,6 +3460,7 @@
       <c r="E285" s="4" t="n"/>
       <c r="F285" s="4" t="n"/>
       <c r="G285" s="4" t="n"/>
+      <c r="H285" s="4" t="n"/>
     </row>
     <row r="286">
       <c r="A286" s="4" t="n"/>
@@ -3176,6 +3470,7 @@
       <c r="E286" s="4" t="n"/>
       <c r="F286" s="4" t="n"/>
       <c r="G286" s="4" t="n"/>
+      <c r="H286" s="4" t="n"/>
     </row>
     <row r="287">
       <c r="A287" s="4" t="n"/>
@@ -3185,6 +3480,7 @@
       <c r="E287" s="4" t="n"/>
       <c r="F287" s="4" t="n"/>
       <c r="G287" s="4" t="n"/>
+      <c r="H287" s="4" t="n"/>
     </row>
     <row r="288">
       <c r="A288" s="4" t="n"/>
@@ -3194,6 +3490,7 @@
       <c r="E288" s="4" t="n"/>
       <c r="F288" s="4" t="n"/>
       <c r="G288" s="4" t="n"/>
+      <c r="H288" s="4" t="n"/>
     </row>
     <row r="289">
       <c r="A289" s="4" t="n"/>
@@ -3203,6 +3500,7 @@
       <c r="E289" s="4" t="n"/>
       <c r="F289" s="4" t="n"/>
       <c r="G289" s="4" t="n"/>
+      <c r="H289" s="4" t="n"/>
     </row>
     <row r="290">
       <c r="A290" s="4" t="n"/>
@@ -3212,6 +3510,7 @@
       <c r="E290" s="4" t="n"/>
       <c r="F290" s="4" t="n"/>
       <c r="G290" s="4" t="n"/>
+      <c r="H290" s="4" t="n"/>
     </row>
     <row r="291">
       <c r="A291" s="4" t="n"/>
@@ -3221,6 +3520,7 @@
       <c r="E291" s="4" t="n"/>
       <c r="F291" s="4" t="n"/>
       <c r="G291" s="4" t="n"/>
+      <c r="H291" s="4" t="n"/>
     </row>
     <row r="292">
       <c r="A292" s="4" t="n"/>
@@ -3230,6 +3530,7 @@
       <c r="E292" s="4" t="n"/>
       <c r="F292" s="4" t="n"/>
       <c r="G292" s="4" t="n"/>
+      <c r="H292" s="4" t="n"/>
     </row>
     <row r="293">
       <c r="A293" s="4" t="n"/>
@@ -3239,6 +3540,7 @@
       <c r="E293" s="4" t="n"/>
       <c r="F293" s="4" t="n"/>
       <c r="G293" s="4" t="n"/>
+      <c r="H293" s="4" t="n"/>
     </row>
     <row r="294">
       <c r="A294" s="4" t="n"/>
@@ -3248,6 +3550,7 @@
       <c r="E294" s="4" t="n"/>
       <c r="F294" s="4" t="n"/>
       <c r="G294" s="4" t="n"/>
+      <c r="H294" s="4" t="n"/>
     </row>
     <row r="295">
       <c r="A295" s="4" t="n"/>
@@ -3257,6 +3560,7 @@
       <c r="E295" s="4" t="n"/>
       <c r="F295" s="4" t="n"/>
       <c r="G295" s="4" t="n"/>
+      <c r="H295" s="4" t="n"/>
     </row>
     <row r="296">
       <c r="A296" s="4" t="n"/>
@@ -3266,6 +3570,7 @@
       <c r="E296" s="4" t="n"/>
       <c r="F296" s="4" t="n"/>
       <c r="G296" s="4" t="n"/>
+      <c r="H296" s="4" t="n"/>
     </row>
     <row r="297">
       <c r="A297" s="4" t="n"/>
@@ -3275,6 +3580,7 @@
       <c r="E297" s="4" t="n"/>
       <c r="F297" s="4" t="n"/>
       <c r="G297" s="4" t="n"/>
+      <c r="H297" s="4" t="n"/>
     </row>
     <row r="298">
       <c r="A298" s="4" t="n"/>
@@ -3284,6 +3590,7 @@
       <c r="E298" s="4" t="n"/>
       <c r="F298" s="4" t="n"/>
       <c r="G298" s="4" t="n"/>
+      <c r="H298" s="4" t="n"/>
     </row>
     <row r="299">
       <c r="A299" s="4" t="n"/>
@@ -3293,6 +3600,7 @@
       <c r="E299" s="4" t="n"/>
       <c r="F299" s="4" t="n"/>
       <c r="G299" s="4" t="n"/>
+      <c r="H299" s="4" t="n"/>
     </row>
     <row r="300">
       <c r="A300" s="4" t="n"/>
@@ -3302,6 +3610,7 @@
       <c r="E300" s="4" t="n"/>
       <c r="F300" s="4" t="n"/>
       <c r="G300" s="4" t="n"/>
+      <c r="H300" s="4" t="n"/>
     </row>
     <row r="301">
       <c r="A301" s="4" t="n"/>
@@ -3311,6 +3620,7 @@
       <c r="E301" s="4" t="n"/>
       <c r="F301" s="4" t="n"/>
       <c r="G301" s="4" t="n"/>
+      <c r="H301" s="4" t="n"/>
     </row>
     <row r="302">
       <c r="A302" s="4" t="n"/>
@@ -3320,6 +3630,7 @@
       <c r="E302" s="4" t="n"/>
       <c r="F302" s="4" t="n"/>
       <c r="G302" s="4" t="n"/>
+      <c r="H302" s="4" t="n"/>
     </row>
     <row r="303">
       <c r="A303" s="4" t="n"/>
@@ -3329,6 +3640,7 @@
       <c r="E303" s="4" t="n"/>
       <c r="F303" s="4" t="n"/>
       <c r="G303" s="4" t="n"/>
+      <c r="H303" s="4" t="n"/>
     </row>
     <row r="304">
       <c r="A304" s="4" t="n"/>
@@ -3338,6 +3650,7 @@
       <c r="E304" s="4" t="n"/>
       <c r="F304" s="4" t="n"/>
       <c r="G304" s="4" t="n"/>
+      <c r="H304" s="4" t="n"/>
     </row>
     <row r="305">
       <c r="A305" s="4" t="n"/>
@@ -3347,6 +3660,7 @@
       <c r="E305" s="4" t="n"/>
       <c r="F305" s="4" t="n"/>
       <c r="G305" s="4" t="n"/>
+      <c r="H305" s="4" t="n"/>
     </row>
     <row r="306">
       <c r="A306" s="4" t="n"/>
@@ -3356,6 +3670,7 @@
       <c r="E306" s="4" t="n"/>
       <c r="F306" s="4" t="n"/>
       <c r="G306" s="4" t="n"/>
+      <c r="H306" s="4" t="n"/>
     </row>
     <row r="307">
       <c r="A307" s="4" t="n"/>
@@ -3365,6 +3680,7 @@
       <c r="E307" s="4" t="n"/>
       <c r="F307" s="4" t="n"/>
       <c r="G307" s="4" t="n"/>
+      <c r="H307" s="4" t="n"/>
     </row>
     <row r="308">
       <c r="A308" s="4" t="n"/>
@@ -3374,6 +3690,7 @@
       <c r="E308" s="4" t="n"/>
       <c r="F308" s="4" t="n"/>
       <c r="G308" s="4" t="n"/>
+      <c r="H308" s="4" t="n"/>
     </row>
     <row r="309">
       <c r="A309" s="4" t="n"/>
@@ -3383,6 +3700,7 @@
       <c r="E309" s="4" t="n"/>
       <c r="F309" s="4" t="n"/>
       <c r="G309" s="4" t="n"/>
+      <c r="H309" s="4" t="n"/>
     </row>
     <row r="310">
       <c r="A310" s="4" t="n"/>
@@ -3392,6 +3710,7 @@
       <c r="E310" s="4" t="n"/>
       <c r="F310" s="4" t="n"/>
       <c r="G310" s="4" t="n"/>
+      <c r="H310" s="4" t="n"/>
     </row>
     <row r="311">
       <c r="A311" s="4" t="n"/>
@@ -3401,6 +3720,7 @@
       <c r="E311" s="4" t="n"/>
       <c r="F311" s="4" t="n"/>
       <c r="G311" s="4" t="n"/>
+      <c r="H311" s="4" t="n"/>
     </row>
     <row r="312">
       <c r="A312" s="4" t="n"/>
@@ -3410,6 +3730,7 @@
       <c r="E312" s="4" t="n"/>
       <c r="F312" s="4" t="n"/>
       <c r="G312" s="4" t="n"/>
+      <c r="H312" s="4" t="n"/>
     </row>
     <row r="313">
       <c r="A313" s="4" t="n"/>
@@ -3419,6 +3740,7 @@
       <c r="E313" s="4" t="n"/>
       <c r="F313" s="4" t="n"/>
       <c r="G313" s="4" t="n"/>
+      <c r="H313" s="4" t="n"/>
     </row>
     <row r="314">
       <c r="A314" s="4" t="n"/>
@@ -3428,6 +3750,7 @@
       <c r="E314" s="4" t="n"/>
       <c r="F314" s="4" t="n"/>
       <c r="G314" s="4" t="n"/>
+      <c r="H314" s="4" t="n"/>
     </row>
     <row r="315">
       <c r="A315" s="4" t="n"/>
@@ -3437,6 +3760,7 @@
       <c r="E315" s="4" t="n"/>
       <c r="F315" s="4" t="n"/>
       <c r="G315" s="4" t="n"/>
+      <c r="H315" s="4" t="n"/>
     </row>
     <row r="316">
       <c r="A316" s="4" t="n"/>
@@ -3446,6 +3770,7 @@
       <c r="E316" s="4" t="n"/>
       <c r="F316" s="4" t="n"/>
       <c r="G316" s="4" t="n"/>
+      <c r="H316" s="4" t="n"/>
     </row>
     <row r="317">
       <c r="A317" s="4" t="n"/>
@@ -3455,6 +3780,7 @@
       <c r="E317" s="4" t="n"/>
       <c r="F317" s="4" t="n"/>
       <c r="G317" s="4" t="n"/>
+      <c r="H317" s="4" t="n"/>
     </row>
     <row r="318">
       <c r="A318" s="4" t="n"/>
@@ -3464,6 +3790,7 @@
       <c r="E318" s="4" t="n"/>
       <c r="F318" s="4" t="n"/>
       <c r="G318" s="4" t="n"/>
+      <c r="H318" s="4" t="n"/>
     </row>
     <row r="319">
       <c r="A319" s="4" t="n"/>
@@ -3473,6 +3800,7 @@
       <c r="E319" s="4" t="n"/>
       <c r="F319" s="4" t="n"/>
       <c r="G319" s="4" t="n"/>
+      <c r="H319" s="4" t="n"/>
     </row>
     <row r="320">
       <c r="A320" s="4" t="n"/>
@@ -3482,6 +3810,7 @@
       <c r="E320" s="4" t="n"/>
       <c r="F320" s="4" t="n"/>
       <c r="G320" s="4" t="n"/>
+      <c r="H320" s="4" t="n"/>
     </row>
     <row r="321">
       <c r="A321" s="4" t="n"/>
@@ -3491,6 +3820,7 @@
       <c r="E321" s="4" t="n"/>
       <c r="F321" s="4" t="n"/>
       <c r="G321" s="4" t="n"/>
+      <c r="H321" s="4" t="n"/>
     </row>
     <row r="322">
       <c r="A322" s="4" t="n"/>
@@ -3500,6 +3830,7 @@
       <c r="E322" s="4" t="n"/>
       <c r="F322" s="4" t="n"/>
       <c r="G322" s="4" t="n"/>
+      <c r="H322" s="4" t="n"/>
     </row>
     <row r="323">
       <c r="A323" s="4" t="n"/>
@@ -3509,6 +3840,7 @@
       <c r="E323" s="4" t="n"/>
       <c r="F323" s="4" t="n"/>
       <c r="G323" s="4" t="n"/>
+      <c r="H323" s="4" t="n"/>
     </row>
     <row r="324">
       <c r="A324" s="4" t="n"/>
@@ -3518,6 +3850,7 @@
       <c r="E324" s="4" t="n"/>
       <c r="F324" s="4" t="n"/>
       <c r="G324" s="4" t="n"/>
+      <c r="H324" s="4" t="n"/>
     </row>
     <row r="325">
       <c r="A325" s="4" t="n"/>
@@ -3527,6 +3860,7 @@
       <c r="E325" s="4" t="n"/>
       <c r="F325" s="4" t="n"/>
       <c r="G325" s="4" t="n"/>
+      <c r="H325" s="4" t="n"/>
     </row>
     <row r="326">
       <c r="A326" s="4" t="n"/>
@@ -3536,6 +3870,7 @@
       <c r="E326" s="4" t="n"/>
       <c r="F326" s="4" t="n"/>
       <c r="G326" s="4" t="n"/>
+      <c r="H326" s="4" t="n"/>
     </row>
     <row r="327">
       <c r="A327" s="4" t="n"/>
@@ -3545,6 +3880,7 @@
       <c r="E327" s="4" t="n"/>
       <c r="F327" s="4" t="n"/>
       <c r="G327" s="4" t="n"/>
+      <c r="H327" s="4" t="n"/>
     </row>
     <row r="328">
       <c r="A328" s="4" t="n"/>
@@ -3554,6 +3890,7 @@
       <c r="E328" s="4" t="n"/>
       <c r="F328" s="4" t="n"/>
       <c r="G328" s="4" t="n"/>
+      <c r="H328" s="4" t="n"/>
     </row>
     <row r="329">
       <c r="A329" s="4" t="n"/>
@@ -3563,6 +3900,7 @@
       <c r="E329" s="4" t="n"/>
       <c r="F329" s="4" t="n"/>
       <c r="G329" s="4" t="n"/>
+      <c r="H329" s="4" t="n"/>
     </row>
     <row r="330">
       <c r="A330" s="4" t="n"/>
@@ -3572,6 +3910,7 @@
       <c r="E330" s="4" t="n"/>
       <c r="F330" s="4" t="n"/>
       <c r="G330" s="4" t="n"/>
+      <c r="H330" s="4" t="n"/>
     </row>
     <row r="331">
       <c r="A331" s="4" t="n"/>
@@ -3581,6 +3920,7 @@
       <c r="E331" s="4" t="n"/>
       <c r="F331" s="4" t="n"/>
       <c r="G331" s="4" t="n"/>
+      <c r="H331" s="4" t="n"/>
     </row>
     <row r="332">
       <c r="A332" s="4" t="n"/>
@@ -3590,6 +3930,7 @@
       <c r="E332" s="4" t="n"/>
       <c r="F332" s="4" t="n"/>
       <c r="G332" s="4" t="n"/>
+      <c r="H332" s="4" t="n"/>
     </row>
     <row r="333">
       <c r="A333" s="4" t="n"/>
@@ -3599,6 +3940,7 @@
       <c r="E333" s="4" t="n"/>
       <c r="F333" s="4" t="n"/>
       <c r="G333" s="4" t="n"/>
+      <c r="H333" s="4" t="n"/>
     </row>
     <row r="334">
       <c r="A334" s="4" t="n"/>
@@ -3608,6 +3950,7 @@
       <c r="E334" s="4" t="n"/>
       <c r="F334" s="4" t="n"/>
       <c r="G334" s="4" t="n"/>
+      <c r="H334" s="4" t="n"/>
     </row>
     <row r="335">
       <c r="A335" s="4" t="n"/>
@@ -3617,6 +3960,7 @@
       <c r="E335" s="4" t="n"/>
       <c r="F335" s="4" t="n"/>
       <c r="G335" s="4" t="n"/>
+      <c r="H335" s="4" t="n"/>
     </row>
     <row r="336">
       <c r="A336" s="4" t="n"/>
@@ -3626,6 +3970,7 @@
       <c r="E336" s="4" t="n"/>
       <c r="F336" s="4" t="n"/>
       <c r="G336" s="4" t="n"/>
+      <c r="H336" s="4" t="n"/>
     </row>
     <row r="337">
       <c r="A337" s="4" t="n"/>
@@ -3635,6 +3980,7 @@
       <c r="E337" s="4" t="n"/>
       <c r="F337" s="4" t="n"/>
       <c r="G337" s="4" t="n"/>
+      <c r="H337" s="4" t="n"/>
     </row>
     <row r="338">
       <c r="A338" s="4" t="n"/>
@@ -3644,6 +3990,7 @@
       <c r="E338" s="4" t="n"/>
       <c r="F338" s="4" t="n"/>
       <c r="G338" s="4" t="n"/>
+      <c r="H338" s="4" t="n"/>
     </row>
     <row r="339">
       <c r="A339" s="4" t="n"/>
@@ -3653,6 +4000,7 @@
       <c r="E339" s="4" t="n"/>
       <c r="F339" s="4" t="n"/>
       <c r="G339" s="4" t="n"/>
+      <c r="H339" s="4" t="n"/>
     </row>
     <row r="340">
       <c r="A340" s="4" t="n"/>
@@ -3662,6 +4010,7 @@
       <c r="E340" s="4" t="n"/>
       <c r="F340" s="4" t="n"/>
       <c r="G340" s="4" t="n"/>
+      <c r="H340" s="4" t="n"/>
     </row>
     <row r="341">
       <c r="A341" s="4" t="n"/>
@@ -3671,6 +4020,7 @@
       <c r="E341" s="4" t="n"/>
       <c r="F341" s="4" t="n"/>
       <c r="G341" s="4" t="n"/>
+      <c r="H341" s="4" t="n"/>
     </row>
     <row r="342">
       <c r="A342" s="4" t="n"/>
@@ -3680,6 +4030,7 @@
       <c r="E342" s="4" t="n"/>
       <c r="F342" s="4" t="n"/>
       <c r="G342" s="4" t="n"/>
+      <c r="H342" s="4" t="n"/>
     </row>
     <row r="343">
       <c r="A343" s="4" t="n"/>
@@ -3689,6 +4040,7 @@
       <c r="E343" s="4" t="n"/>
       <c r="F343" s="4" t="n"/>
       <c r="G343" s="4" t="n"/>
+      <c r="H343" s="4" t="n"/>
     </row>
     <row r="344">
       <c r="A344" s="4" t="n"/>
@@ -3698,6 +4050,7 @@
       <c r="E344" s="4" t="n"/>
       <c r="F344" s="4" t="n"/>
       <c r="G344" s="4" t="n"/>
+      <c r="H344" s="4" t="n"/>
     </row>
     <row r="345">
       <c r="A345" s="4" t="n"/>
@@ -3707,6 +4060,7 @@
       <c r="E345" s="4" t="n"/>
       <c r="F345" s="4" t="n"/>
       <c r="G345" s="4" t="n"/>
+      <c r="H345" s="4" t="n"/>
     </row>
     <row r="346">
       <c r="A346" s="4" t="n"/>
@@ -3716,6 +4070,7 @@
       <c r="E346" s="4" t="n"/>
       <c r="F346" s="4" t="n"/>
       <c r="G346" s="4" t="n"/>
+      <c r="H346" s="4" t="n"/>
     </row>
     <row r="347">
       <c r="A347" s="4" t="n"/>
@@ -3725,6 +4080,7 @@
       <c r="E347" s="4" t="n"/>
       <c r="F347" s="4" t="n"/>
       <c r="G347" s="4" t="n"/>
+      <c r="H347" s="4" t="n"/>
     </row>
     <row r="348">
       <c r="A348" s="4" t="n"/>
@@ -3734,6 +4090,7 @@
       <c r="E348" s="4" t="n"/>
       <c r="F348" s="4" t="n"/>
       <c r="G348" s="4" t="n"/>
+      <c r="H348" s="4" t="n"/>
     </row>
     <row r="349">
       <c r="A349" s="4" t="n"/>
@@ -3743,6 +4100,7 @@
       <c r="E349" s="4" t="n"/>
       <c r="F349" s="4" t="n"/>
       <c r="G349" s="4" t="n"/>
+      <c r="H349" s="4" t="n"/>
     </row>
     <row r="350">
       <c r="A350" s="4" t="n"/>
@@ -3752,6 +4110,7 @@
       <c r="E350" s="4" t="n"/>
       <c r="F350" s="4" t="n"/>
       <c r="G350" s="4" t="n"/>
+      <c r="H350" s="4" t="n"/>
     </row>
     <row r="351">
       <c r="A351" s="4" t="n"/>
@@ -3761,6 +4120,7 @@
       <c r="E351" s="4" t="n"/>
       <c r="F351" s="4" t="n"/>
       <c r="G351" s="4" t="n"/>
+      <c r="H351" s="4" t="n"/>
     </row>
     <row r="352">
       <c r="A352" s="4" t="n"/>
@@ -3770,6 +4130,7 @@
       <c r="E352" s="4" t="n"/>
       <c r="F352" s="4" t="n"/>
       <c r="G352" s="4" t="n"/>
+      <c r="H352" s="4" t="n"/>
     </row>
     <row r="353">
       <c r="A353" s="4" t="n"/>
@@ -3779,6 +4140,7 @@
       <c r="E353" s="4" t="n"/>
       <c r="F353" s="4" t="n"/>
       <c r="G353" s="4" t="n"/>
+      <c r="H353" s="4" t="n"/>
     </row>
     <row r="354">
       <c r="A354" s="4" t="n"/>
@@ -3788,6 +4150,7 @@
       <c r="E354" s="4" t="n"/>
       <c r="F354" s="4" t="n"/>
       <c r="G354" s="4" t="n"/>
+      <c r="H354" s="4" t="n"/>
     </row>
     <row r="355">
       <c r="A355" s="4" t="n"/>
@@ -3797,6 +4160,7 @@
       <c r="E355" s="4" t="n"/>
       <c r="F355" s="4" t="n"/>
       <c r="G355" s="4" t="n"/>
+      <c r="H355" s="4" t="n"/>
     </row>
     <row r="356">
       <c r="A356" s="4" t="n"/>
@@ -3806,6 +4170,7 @@
       <c r="E356" s="4" t="n"/>
       <c r="F356" s="4" t="n"/>
       <c r="G356" s="4" t="n"/>
+      <c r="H356" s="4" t="n"/>
     </row>
     <row r="357">
       <c r="A357" s="4" t="n"/>
@@ -3815,6 +4180,7 @@
       <c r="E357" s="4" t="n"/>
       <c r="F357" s="4" t="n"/>
       <c r="G357" s="4" t="n"/>
+      <c r="H357" s="4" t="n"/>
     </row>
     <row r="358">
       <c r="A358" s="4" t="n"/>
@@ -3824,6 +4190,7 @@
       <c r="E358" s="4" t="n"/>
       <c r="F358" s="4" t="n"/>
       <c r="G358" s="4" t="n"/>
+      <c r="H358" s="4" t="n"/>
     </row>
     <row r="359">
       <c r="A359" s="4" t="n"/>
@@ -3833,6 +4200,7 @@
       <c r="E359" s="4" t="n"/>
       <c r="F359" s="4" t="n"/>
       <c r="G359" s="4" t="n"/>
+      <c r="H359" s="4" t="n"/>
     </row>
     <row r="360">
       <c r="A360" s="4" t="n"/>
@@ -3842,6 +4210,7 @@
       <c r="E360" s="4" t="n"/>
       <c r="F360" s="4" t="n"/>
       <c r="G360" s="4" t="n"/>
+      <c r="H360" s="4" t="n"/>
     </row>
     <row r="361">
       <c r="A361" s="4" t="n"/>
@@ -3851,6 +4220,7 @@
       <c r="E361" s="4" t="n"/>
       <c r="F361" s="4" t="n"/>
       <c r="G361" s="4" t="n"/>
+      <c r="H361" s="4" t="n"/>
     </row>
     <row r="362">
       <c r="A362" s="4" t="n"/>
@@ -3860,6 +4230,7 @@
       <c r="E362" s="4" t="n"/>
       <c r="F362" s="4" t="n"/>
       <c r="G362" s="4" t="n"/>
+      <c r="H362" s="4" t="n"/>
     </row>
     <row r="363">
       <c r="A363" s="4" t="n"/>
@@ -3869,6 +4240,7 @@
       <c r="E363" s="4" t="n"/>
       <c r="F363" s="4" t="n"/>
       <c r="G363" s="4" t="n"/>
+      <c r="H363" s="4" t="n"/>
     </row>
     <row r="364">
       <c r="A364" s="4" t="n"/>
@@ -3878,6 +4250,7 @@
       <c r="E364" s="4" t="n"/>
       <c r="F364" s="4" t="n"/>
       <c r="G364" s="4" t="n"/>
+      <c r="H364" s="4" t="n"/>
     </row>
     <row r="365">
       <c r="A365" s="4" t="n"/>
@@ -3887,6 +4260,7 @@
       <c r="E365" s="4" t="n"/>
       <c r="F365" s="4" t="n"/>
       <c r="G365" s="4" t="n"/>
+      <c r="H365" s="4" t="n"/>
     </row>
     <row r="366">
       <c r="A366" s="4" t="n"/>
@@ -3896,6 +4270,7 @@
       <c r="E366" s="4" t="n"/>
       <c r="F366" s="4" t="n"/>
       <c r="G366" s="4" t="n"/>
+      <c r="H366" s="4" t="n"/>
     </row>
     <row r="367">
       <c r="A367" s="4" t="n"/>
@@ -3905,6 +4280,7 @@
       <c r="E367" s="4" t="n"/>
       <c r="F367" s="4" t="n"/>
       <c r="G367" s="4" t="n"/>
+      <c r="H367" s="4" t="n"/>
     </row>
     <row r="368">
       <c r="A368" s="4" t="n"/>
@@ -3914,6 +4290,7 @@
       <c r="E368" s="4" t="n"/>
       <c r="F368" s="4" t="n"/>
       <c r="G368" s="4" t="n"/>
+      <c r="H368" s="4" t="n"/>
     </row>
     <row r="369">
       <c r="A369" s="4" t="n"/>
@@ -3923,6 +4300,7 @@
       <c r="E369" s="4" t="n"/>
       <c r="F369" s="4" t="n"/>
       <c r="G369" s="4" t="n"/>
+      <c r="H369" s="4" t="n"/>
     </row>
     <row r="370">
       <c r="A370" s="4" t="n"/>
@@ -3932,6 +4310,7 @@
       <c r="E370" s="4" t="n"/>
       <c r="F370" s="4" t="n"/>
       <c r="G370" s="4" t="n"/>
+      <c r="H370" s="4" t="n"/>
     </row>
     <row r="371">
       <c r="A371" s="4" t="n"/>
@@ -3941,6 +4320,7 @@
       <c r="E371" s="4" t="n"/>
       <c r="F371" s="4" t="n"/>
       <c r="G371" s="4" t="n"/>
+      <c r="H371" s="4" t="n"/>
     </row>
     <row r="372">
       <c r="A372" s="4" t="n"/>
@@ -3950,6 +4330,7 @@
       <c r="E372" s="4" t="n"/>
       <c r="F372" s="4" t="n"/>
       <c r="G372" s="4" t="n"/>
+      <c r="H372" s="4" t="n"/>
     </row>
     <row r="373">
       <c r="A373" s="4" t="n"/>
@@ -3959,6 +4340,7 @@
       <c r="E373" s="4" t="n"/>
       <c r="F373" s="4" t="n"/>
       <c r="G373" s="4" t="n"/>
+      <c r="H373" s="4" t="n"/>
     </row>
     <row r="374">
       <c r="A374" s="4" t="n"/>
@@ -3968,6 +4350,7 @@
       <c r="E374" s="4" t="n"/>
       <c r="F374" s="4" t="n"/>
       <c r="G374" s="4" t="n"/>
+      <c r="H374" s="4" t="n"/>
     </row>
     <row r="375">
       <c r="A375" s="4" t="n"/>
@@ -3977,6 +4360,7 @@
       <c r="E375" s="4" t="n"/>
       <c r="F375" s="4" t="n"/>
       <c r="G375" s="4" t="n"/>
+      <c r="H375" s="4" t="n"/>
     </row>
     <row r="376">
       <c r="A376" s="4" t="n"/>
@@ -3986,6 +4370,7 @@
       <c r="E376" s="4" t="n"/>
       <c r="F376" s="4" t="n"/>
       <c r="G376" s="4" t="n"/>
+      <c r="H376" s="4" t="n"/>
     </row>
     <row r="377">
       <c r="A377" s="4" t="n"/>
@@ -3995,6 +4380,7 @@
       <c r="E377" s="4" t="n"/>
       <c r="F377" s="4" t="n"/>
       <c r="G377" s="4" t="n"/>
+      <c r="H377" s="4" t="n"/>
     </row>
     <row r="378">
       <c r="A378" s="4" t="n"/>
@@ -4004,6 +4390,7 @@
       <c r="E378" s="4" t="n"/>
       <c r="F378" s="4" t="n"/>
       <c r="G378" s="4" t="n"/>
+      <c r="H378" s="4" t="n"/>
     </row>
     <row r="379">
       <c r="A379" s="4" t="n"/>
@@ -4013,6 +4400,7 @@
       <c r="E379" s="4" t="n"/>
       <c r="F379" s="4" t="n"/>
       <c r="G379" s="4" t="n"/>
+      <c r="H379" s="4" t="n"/>
     </row>
     <row r="380">
       <c r="A380" s="4" t="n"/>
@@ -4022,6 +4410,7 @@
       <c r="E380" s="4" t="n"/>
       <c r="F380" s="4" t="n"/>
       <c r="G380" s="4" t="n"/>
+      <c r="H380" s="4" t="n"/>
     </row>
     <row r="381">
       <c r="A381" s="4" t="n"/>
@@ -4031,6 +4420,7 @@
       <c r="E381" s="4" t="n"/>
       <c r="F381" s="4" t="n"/>
       <c r="G381" s="4" t="n"/>
+      <c r="H381" s="4" t="n"/>
     </row>
     <row r="382">
       <c r="A382" s="4" t="n"/>
@@ -4040,6 +4430,7 @@
       <c r="E382" s="4" t="n"/>
       <c r="F382" s="4" t="n"/>
       <c r="G382" s="4" t="n"/>
+      <c r="H382" s="4" t="n"/>
     </row>
     <row r="383">
       <c r="A383" s="4" t="n"/>
@@ -4049,6 +4440,7 @@
       <c r="E383" s="4" t="n"/>
       <c r="F383" s="4" t="n"/>
       <c r="G383" s="4" t="n"/>
+      <c r="H383" s="4" t="n"/>
     </row>
     <row r="384">
       <c r="A384" s="4" t="n"/>
@@ -4058,6 +4450,7 @@
       <c r="E384" s="4" t="n"/>
       <c r="F384" s="4" t="n"/>
       <c r="G384" s="4" t="n"/>
+      <c r="H384" s="4" t="n"/>
     </row>
     <row r="385">
       <c r="A385" s="4" t="n"/>
@@ -4067,6 +4460,7 @@
       <c r="E385" s="4" t="n"/>
       <c r="F385" s="4" t="n"/>
       <c r="G385" s="4" t="n"/>
+      <c r="H385" s="4" t="n"/>
     </row>
     <row r="386">
       <c r="A386" s="4" t="n"/>
@@ -4076,6 +4470,7 @@
       <c r="E386" s="4" t="n"/>
       <c r="F386" s="4" t="n"/>
       <c r="G386" s="4" t="n"/>
+      <c r="H386" s="4" t="n"/>
     </row>
     <row r="387">
       <c r="A387" s="4" t="n"/>
@@ -4085,6 +4480,7 @@
       <c r="E387" s="4" t="n"/>
       <c r="F387" s="4" t="n"/>
       <c r="G387" s="4" t="n"/>
+      <c r="H387" s="4" t="n"/>
     </row>
     <row r="388">
       <c r="A388" s="4" t="n"/>
@@ -4094,6 +4490,7 @@
       <c r="E388" s="4" t="n"/>
       <c r="F388" s="4" t="n"/>
       <c r="G388" s="4" t="n"/>
+      <c r="H388" s="4" t="n"/>
     </row>
     <row r="389">
       <c r="A389" s="4" t="n"/>
@@ -4103,6 +4500,7 @@
       <c r="E389" s="4" t="n"/>
       <c r="F389" s="4" t="n"/>
       <c r="G389" s="4" t="n"/>
+      <c r="H389" s="4" t="n"/>
     </row>
     <row r="390">
       <c r="A390" s="4" t="n"/>
@@ -4112,6 +4510,7 @@
       <c r="E390" s="4" t="n"/>
       <c r="F390" s="4" t="n"/>
       <c r="G390" s="4" t="n"/>
+      <c r="H390" s="4" t="n"/>
     </row>
     <row r="391">
       <c r="A391" s="4" t="n"/>
@@ -4121,6 +4520,7 @@
       <c r="E391" s="4" t="n"/>
       <c r="F391" s="4" t="n"/>
       <c r="G391" s="4" t="n"/>
+      <c r="H391" s="4" t="n"/>
     </row>
     <row r="392">
       <c r="A392" s="4" t="n"/>
@@ -4130,6 +4530,7 @@
       <c r="E392" s="4" t="n"/>
       <c r="F392" s="4" t="n"/>
       <c r="G392" s="4" t="n"/>
+      <c r="H392" s="4" t="n"/>
     </row>
     <row r="393">
       <c r="A393" s="4" t="n"/>
@@ -4139,6 +4540,7 @@
       <c r="E393" s="4" t="n"/>
       <c r="F393" s="4" t="n"/>
       <c r="G393" s="4" t="n"/>
+      <c r="H393" s="4" t="n"/>
     </row>
     <row r="394">
       <c r="A394" s="4" t="n"/>
@@ -4148,6 +4550,7 @@
       <c r="E394" s="4" t="n"/>
       <c r="F394" s="4" t="n"/>
       <c r="G394" s="4" t="n"/>
+      <c r="H394" s="4" t="n"/>
     </row>
     <row r="395">
       <c r="A395" s="4" t="n"/>
@@ -4157,6 +4560,7 @@
       <c r="E395" s="4" t="n"/>
       <c r="F395" s="4" t="n"/>
       <c r="G395" s="4" t="n"/>
+      <c r="H395" s="4" t="n"/>
     </row>
     <row r="396">
       <c r="A396" s="4" t="n"/>
@@ -4166,6 +4570,7 @@
       <c r="E396" s="4" t="n"/>
       <c r="F396" s="4" t="n"/>
       <c r="G396" s="4" t="n"/>
+      <c r="H396" s="4" t="n"/>
     </row>
     <row r="397">
       <c r="A397" s="4" t="n"/>
@@ -4175,6 +4580,7 @@
       <c r="E397" s="4" t="n"/>
       <c r="F397" s="4" t="n"/>
       <c r="G397" s="4" t="n"/>
+      <c r="H397" s="4" t="n"/>
     </row>
     <row r="398">
       <c r="A398" s="4" t="n"/>
@@ -4184,6 +4590,7 @@
       <c r="E398" s="4" t="n"/>
       <c r="F398" s="4" t="n"/>
       <c r="G398" s="4" t="n"/>
+      <c r="H398" s="4" t="n"/>
     </row>
     <row r="399">
       <c r="A399" s="4" t="n"/>
@@ -4193,6 +4600,7 @@
       <c r="E399" s="4" t="n"/>
       <c r="F399" s="4" t="n"/>
       <c r="G399" s="4" t="n"/>
+      <c r="H399" s="4" t="n"/>
     </row>
     <row r="400">
       <c r="A400" s="4" t="n"/>
@@ -4202,6 +4610,7 @@
       <c r="E400" s="4" t="n"/>
       <c r="F400" s="4" t="n"/>
       <c r="G400" s="4" t="n"/>
+      <c r="H400" s="4" t="n"/>
     </row>
     <row r="401">
       <c r="A401" s="4" t="n"/>
@@ -4211,6 +4620,7 @@
       <c r="E401" s="4" t="n"/>
       <c r="F401" s="4" t="n"/>
       <c r="G401" s="4" t="n"/>
+      <c r="H401" s="4" t="n"/>
     </row>
     <row r="402">
       <c r="A402" s="4" t="n"/>
@@ -4220,6 +4630,7 @@
       <c r="E402" s="4" t="n"/>
       <c r="F402" s="4" t="n"/>
       <c r="G402" s="4" t="n"/>
+      <c r="H402" s="4" t="n"/>
     </row>
     <row r="403">
       <c r="A403" s="4" t="n"/>
@@ -4229,6 +4640,7 @@
       <c r="E403" s="4" t="n"/>
       <c r="F403" s="4" t="n"/>
       <c r="G403" s="4" t="n"/>
+      <c r="H403" s="4" t="n"/>
     </row>
     <row r="404">
       <c r="A404" s="4" t="n"/>
@@ -4238,6 +4650,7 @@
       <c r="E404" s="4" t="n"/>
       <c r="F404" s="4" t="n"/>
       <c r="G404" s="4" t="n"/>
+      <c r="H404" s="4" t="n"/>
     </row>
     <row r="405">
       <c r="A405" s="4" t="n"/>
@@ -4247,6 +4660,7 @@
       <c r="E405" s="4" t="n"/>
       <c r="F405" s="4" t="n"/>
       <c r="G405" s="4" t="n"/>
+      <c r="H405" s="4" t="n"/>
     </row>
     <row r="406">
       <c r="A406" s="4" t="n"/>
@@ -4256,6 +4670,7 @@
       <c r="E406" s="4" t="n"/>
       <c r="F406" s="4" t="n"/>
       <c r="G406" s="4" t="n"/>
+      <c r="H406" s="4" t="n"/>
     </row>
     <row r="407">
       <c r="A407" s="4" t="n"/>
@@ -4265,6 +4680,7 @@
       <c r="E407" s="4" t="n"/>
       <c r="F407" s="4" t="n"/>
       <c r="G407" s="4" t="n"/>
+      <c r="H407" s="4" t="n"/>
     </row>
     <row r="408">
       <c r="A408" s="4" t="n"/>
@@ -4274,6 +4690,7 @@
       <c r="E408" s="4" t="n"/>
       <c r="F408" s="4" t="n"/>
       <c r="G408" s="4" t="n"/>
+      <c r="H408" s="4" t="n"/>
     </row>
     <row r="409">
       <c r="A409" s="4" t="n"/>
@@ -4283,6 +4700,7 @@
       <c r="E409" s="4" t="n"/>
       <c r="F409" s="4" t="n"/>
       <c r="G409" s="4" t="n"/>
+      <c r="H409" s="4" t="n"/>
     </row>
     <row r="410">
       <c r="A410" s="4" t="n"/>
@@ -4292,6 +4710,7 @@
       <c r="E410" s="4" t="n"/>
       <c r="F410" s="4" t="n"/>
       <c r="G410" s="4" t="n"/>
+      <c r="H410" s="4" t="n"/>
     </row>
     <row r="411">
       <c r="A411" s="4" t="n"/>
@@ -4301,6 +4720,7 @@
       <c r="E411" s="4" t="n"/>
       <c r="F411" s="4" t="n"/>
       <c r="G411" s="4" t="n"/>
+      <c r="H411" s="4" t="n"/>
     </row>
     <row r="412">
       <c r="A412" s="4" t="n"/>
@@ -4310,6 +4730,7 @@
       <c r="E412" s="4" t="n"/>
       <c r="F412" s="4" t="n"/>
       <c r="G412" s="4" t="n"/>
+      <c r="H412" s="4" t="n"/>
     </row>
     <row r="413">
       <c r="A413" s="4" t="n"/>
@@ -4319,6 +4740,7 @@
       <c r="E413" s="4" t="n"/>
       <c r="F413" s="4" t="n"/>
       <c r="G413" s="4" t="n"/>
+      <c r="H413" s="4" t="n"/>
     </row>
     <row r="414">
       <c r="A414" s="4" t="n"/>
@@ -4328,6 +4750,7 @@
       <c r="E414" s="4" t="n"/>
       <c r="F414" s="4" t="n"/>
       <c r="G414" s="4" t="n"/>
+      <c r="H414" s="4" t="n"/>
     </row>
     <row r="415">
       <c r="A415" s="4" t="n"/>
@@ -4337,6 +4760,7 @@
       <c r="E415" s="4" t="n"/>
       <c r="F415" s="4" t="n"/>
       <c r="G415" s="4" t="n"/>
+      <c r="H415" s="4" t="n"/>
     </row>
     <row r="416">
       <c r="A416" s="4" t="n"/>
@@ -4346,6 +4770,7 @@
       <c r="E416" s="4" t="n"/>
       <c r="F416" s="4" t="n"/>
       <c r="G416" s="4" t="n"/>
+      <c r="H416" s="4" t="n"/>
     </row>
     <row r="417">
       <c r="A417" s="4" t="n"/>
@@ -4355,6 +4780,7 @@
       <c r="E417" s="4" t="n"/>
       <c r="F417" s="4" t="n"/>
       <c r="G417" s="4" t="n"/>
+      <c r="H417" s="4" t="n"/>
     </row>
     <row r="418">
       <c r="A418" s="4" t="n"/>
@@ -4364,6 +4790,7 @@
       <c r="E418" s="4" t="n"/>
       <c r="F418" s="4" t="n"/>
       <c r="G418" s="4" t="n"/>
+      <c r="H418" s="4" t="n"/>
     </row>
     <row r="419">
       <c r="A419" s="4" t="n"/>
@@ -4373,6 +4800,7 @@
       <c r="E419" s="4" t="n"/>
       <c r="F419" s="4" t="n"/>
       <c r="G419" s="4" t="n"/>
+      <c r="H419" s="4" t="n"/>
     </row>
     <row r="420">
       <c r="A420" s="4" t="n"/>
@@ -4382,6 +4810,7 @@
       <c r="E420" s="4" t="n"/>
       <c r="F420" s="4" t="n"/>
       <c r="G420" s="4" t="n"/>
+      <c r="H420" s="4" t="n"/>
     </row>
     <row r="421">
       <c r="A421" s="4" t="n"/>
@@ -4391,6 +4820,7 @@
       <c r="E421" s="4" t="n"/>
       <c r="F421" s="4" t="n"/>
       <c r="G421" s="4" t="n"/>
+      <c r="H421" s="4" t="n"/>
     </row>
     <row r="422">
       <c r="A422" s="4" t="n"/>
@@ -4400,6 +4830,7 @@
       <c r="E422" s="4" t="n"/>
       <c r="F422" s="4" t="n"/>
       <c r="G422" s="4" t="n"/>
+      <c r="H422" s="4" t="n"/>
     </row>
     <row r="423">
       <c r="A423" s="4" t="n"/>
@@ -4409,6 +4840,7 @@
       <c r="E423" s="4" t="n"/>
       <c r="F423" s="4" t="n"/>
       <c r="G423" s="4" t="n"/>
+      <c r="H423" s="4" t="n"/>
     </row>
     <row r="424">
       <c r="A424" s="4" t="n"/>
@@ -4418,6 +4850,7 @@
       <c r="E424" s="4" t="n"/>
       <c r="F424" s="4" t="n"/>
       <c r="G424" s="4" t="n"/>
+      <c r="H424" s="4" t="n"/>
     </row>
     <row r="425">
       <c r="A425" s="4" t="n"/>
@@ -4427,6 +4860,7 @@
       <c r="E425" s="4" t="n"/>
       <c r="F425" s="4" t="n"/>
       <c r="G425" s="4" t="n"/>
+      <c r="H425" s="4" t="n"/>
     </row>
     <row r="426">
       <c r="A426" s="4" t="n"/>
@@ -4436,6 +4870,7 @@
       <c r="E426" s="4" t="n"/>
       <c r="F426" s="4" t="n"/>
       <c r="G426" s="4" t="n"/>
+      <c r="H426" s="4" t="n"/>
     </row>
     <row r="427">
       <c r="A427" s="4" t="n"/>
@@ -4445,6 +4880,7 @@
       <c r="E427" s="4" t="n"/>
       <c r="F427" s="4" t="n"/>
       <c r="G427" s="4" t="n"/>
+      <c r="H427" s="4" t="n"/>
     </row>
     <row r="428">
       <c r="A428" s="4" t="n"/>
@@ -4454,6 +4890,7 @@
       <c r="E428" s="4" t="n"/>
       <c r="F428" s="4" t="n"/>
       <c r="G428" s="4" t="n"/>
+      <c r="H428" s="4" t="n"/>
     </row>
     <row r="429">
       <c r="A429" s="4" t="n"/>
@@ -4463,6 +4900,7 @@
       <c r="E429" s="4" t="n"/>
       <c r="F429" s="4" t="n"/>
       <c r="G429" s="4" t="n"/>
+      <c r="H429" s="4" t="n"/>
     </row>
     <row r="430">
       <c r="A430" s="4" t="n"/>
@@ -4472,6 +4910,7 @@
       <c r="E430" s="4" t="n"/>
       <c r="F430" s="4" t="n"/>
       <c r="G430" s="4" t="n"/>
+      <c r="H430" s="4" t="n"/>
     </row>
     <row r="431">
       <c r="A431" s="4" t="n"/>
@@ -4481,6 +4920,7 @@
       <c r="E431" s="4" t="n"/>
       <c r="F431" s="4" t="n"/>
       <c r="G431" s="4" t="n"/>
+      <c r="H431" s="4" t="n"/>
     </row>
     <row r="432">
       <c r="A432" s="4" t="n"/>
@@ -4490,6 +4930,7 @@
       <c r="E432" s="4" t="n"/>
       <c r="F432" s="4" t="n"/>
       <c r="G432" s="4" t="n"/>
+      <c r="H432" s="4" t="n"/>
     </row>
     <row r="433">
       <c r="A433" s="4" t="n"/>
@@ -4499,6 +4940,7 @@
       <c r="E433" s="4" t="n"/>
       <c r="F433" s="4" t="n"/>
       <c r="G433" s="4" t="n"/>
+      <c r="H433" s="4" t="n"/>
     </row>
     <row r="434">
       <c r="A434" s="4" t="n"/>
@@ -4508,6 +4950,7 @@
       <c r="E434" s="4" t="n"/>
       <c r="F434" s="4" t="n"/>
       <c r="G434" s="4" t="n"/>
+      <c r="H434" s="4" t="n"/>
     </row>
     <row r="435">
       <c r="A435" s="4" t="n"/>
@@ -4517,6 +4960,7 @@
       <c r="E435" s="4" t="n"/>
       <c r="F435" s="4" t="n"/>
       <c r="G435" s="4" t="n"/>
+      <c r="H435" s="4" t="n"/>
     </row>
     <row r="436">
       <c r="A436" s="4" t="n"/>
@@ -4526,6 +4970,7 @@
       <c r="E436" s="4" t="n"/>
       <c r="F436" s="4" t="n"/>
       <c r="G436" s="4" t="n"/>
+      <c r="H436" s="4" t="n"/>
     </row>
     <row r="437">
       <c r="A437" s="4" t="n"/>
@@ -4535,6 +4980,7 @@
       <c r="E437" s="4" t="n"/>
       <c r="F437" s="4" t="n"/>
       <c r="G437" s="4" t="n"/>
+      <c r="H437" s="4" t="n"/>
     </row>
     <row r="438">
       <c r="A438" s="4" t="n"/>
@@ -4544,6 +4990,7 @@
       <c r="E438" s="4" t="n"/>
       <c r="F438" s="4" t="n"/>
       <c r="G438" s="4" t="n"/>
+      <c r="H438" s="4" t="n"/>
     </row>
     <row r="439">
       <c r="A439" s="4" t="n"/>
@@ -4553,6 +5000,7 @@
       <c r="E439" s="4" t="n"/>
       <c r="F439" s="4" t="n"/>
       <c r="G439" s="4" t="n"/>
+      <c r="H439" s="4" t="n"/>
     </row>
     <row r="440">
       <c r="A440" s="4" t="n"/>
@@ -4562,6 +5010,7 @@
       <c r="E440" s="4" t="n"/>
       <c r="F440" s="4" t="n"/>
       <c r="G440" s="4" t="n"/>
+      <c r="H440" s="4" t="n"/>
     </row>
     <row r="441">
       <c r="A441" s="4" t="n"/>
@@ -4571,6 +5020,7 @@
       <c r="E441" s="4" t="n"/>
       <c r="F441" s="4" t="n"/>
       <c r="G441" s="4" t="n"/>
+      <c r="H441" s="4" t="n"/>
     </row>
     <row r="442">
       <c r="A442" s="4" t="n"/>
@@ -4580,6 +5030,7 @@
       <c r="E442" s="4" t="n"/>
       <c r="F442" s="4" t="n"/>
       <c r="G442" s="4" t="n"/>
+      <c r="H442" s="4" t="n"/>
     </row>
     <row r="443">
       <c r="A443" s="4" t="n"/>
@@ -4589,6 +5040,7 @@
       <c r="E443" s="4" t="n"/>
       <c r="F443" s="4" t="n"/>
       <c r="G443" s="4" t="n"/>
+      <c r="H443" s="4" t="n"/>
     </row>
     <row r="444">
       <c r="A444" s="4" t="n"/>
@@ -4598,6 +5050,7 @@
       <c r="E444" s="4" t="n"/>
       <c r="F444" s="4" t="n"/>
       <c r="G444" s="4" t="n"/>
+      <c r="H444" s="4" t="n"/>
     </row>
     <row r="445">
       <c r="A445" s="4" t="n"/>
@@ -4607,6 +5060,7 @@
       <c r="E445" s="4" t="n"/>
       <c r="F445" s="4" t="n"/>
       <c r="G445" s="4" t="n"/>
+      <c r="H445" s="4" t="n"/>
     </row>
     <row r="446">
       <c r="A446" s="4" t="n"/>
@@ -4616,6 +5070,7 @@
       <c r="E446" s="4" t="n"/>
       <c r="F446" s="4" t="n"/>
       <c r="G446" s="4" t="n"/>
+      <c r="H446" s="4" t="n"/>
     </row>
     <row r="447">
       <c r="A447" s="4" t="n"/>
@@ -4625,6 +5080,7 @@
       <c r="E447" s="4" t="n"/>
       <c r="F447" s="4" t="n"/>
       <c r="G447" s="4" t="n"/>
+      <c r="H447" s="4" t="n"/>
     </row>
     <row r="448">
       <c r="A448" s="4" t="n"/>
@@ -4634,6 +5090,7 @@
       <c r="E448" s="4" t="n"/>
       <c r="F448" s="4" t="n"/>
       <c r="G448" s="4" t="n"/>
+      <c r="H448" s="4" t="n"/>
     </row>
     <row r="449">
       <c r="A449" s="4" t="n"/>
@@ -4643,6 +5100,7 @@
       <c r="E449" s="4" t="n"/>
       <c r="F449" s="4" t="n"/>
       <c r="G449" s="4" t="n"/>
+      <c r="H449" s="4" t="n"/>
     </row>
     <row r="450">
       <c r="A450" s="4" t="n"/>
@@ -4652,6 +5110,7 @@
       <c r="E450" s="4" t="n"/>
       <c r="F450" s="4" t="n"/>
       <c r="G450" s="4" t="n"/>
+      <c r="H450" s="4" t="n"/>
     </row>
     <row r="451">
       <c r="A451" s="4" t="n"/>
@@ -4661,6 +5120,7 @@
       <c r="E451" s="4" t="n"/>
       <c r="F451" s="4" t="n"/>
       <c r="G451" s="4" t="n"/>
+      <c r="H451" s="4" t="n"/>
     </row>
     <row r="452">
       <c r="A452" s="4" t="n"/>
@@ -4670,6 +5130,7 @@
       <c r="E452" s="4" t="n"/>
       <c r="F452" s="4" t="n"/>
       <c r="G452" s="4" t="n"/>
+      <c r="H452" s="4" t="n"/>
     </row>
     <row r="453">
       <c r="A453" s="4" t="n"/>
@@ -4679,6 +5140,7 @@
       <c r="E453" s="4" t="n"/>
       <c r="F453" s="4" t="n"/>
       <c r="G453" s="4" t="n"/>
+      <c r="H453" s="4" t="n"/>
     </row>
     <row r="454">
       <c r="A454" s="4" t="n"/>
@@ -4688,6 +5150,7 @@
       <c r="E454" s="4" t="n"/>
       <c r="F454" s="4" t="n"/>
       <c r="G454" s="4" t="n"/>
+      <c r="H454" s="4" t="n"/>
     </row>
     <row r="455">
       <c r="A455" s="4" t="n"/>
@@ -4697,6 +5160,7 @@
       <c r="E455" s="4" t="n"/>
       <c r="F455" s="4" t="n"/>
       <c r="G455" s="4" t="n"/>
+      <c r="H455" s="4" t="n"/>
     </row>
     <row r="456">
       <c r="A456" s="4" t="n"/>
@@ -4706,6 +5170,7 @@
       <c r="E456" s="4" t="n"/>
       <c r="F456" s="4" t="n"/>
       <c r="G456" s="4" t="n"/>
+      <c r="H456" s="4" t="n"/>
     </row>
     <row r="457">
       <c r="A457" s="4" t="n"/>
@@ -4715,6 +5180,7 @@
       <c r="E457" s="4" t="n"/>
       <c r="F457" s="4" t="n"/>
       <c r="G457" s="4" t="n"/>
+      <c r="H457" s="4" t="n"/>
     </row>
     <row r="458">
       <c r="A458" s="4" t="n"/>
@@ -4724,6 +5190,7 @@
       <c r="E458" s="4" t="n"/>
       <c r="F458" s="4" t="n"/>
       <c r="G458" s="4" t="n"/>
+      <c r="H458" s="4" t="n"/>
     </row>
     <row r="459">
       <c r="A459" s="4" t="n"/>
@@ -4733,6 +5200,7 @@
       <c r="E459" s="4" t="n"/>
       <c r="F459" s="4" t="n"/>
       <c r="G459" s="4" t="n"/>
+      <c r="H459" s="4" t="n"/>
     </row>
     <row r="460">
       <c r="A460" s="4" t="n"/>
@@ -4742,6 +5210,7 @@
       <c r="E460" s="4" t="n"/>
       <c r="F460" s="4" t="n"/>
       <c r="G460" s="4" t="n"/>
+      <c r="H460" s="4" t="n"/>
     </row>
     <row r="461">
       <c r="A461" s="4" t="n"/>
@@ -4751,6 +5220,7 @@
       <c r="E461" s="4" t="n"/>
       <c r="F461" s="4" t="n"/>
       <c r="G461" s="4" t="n"/>
+      <c r="H461" s="4" t="n"/>
     </row>
     <row r="462">
       <c r="A462" s="4" t="n"/>
@@ -4760,6 +5230,7 @@
       <c r="E462" s="4" t="n"/>
       <c r="F462" s="4" t="n"/>
       <c r="G462" s="4" t="n"/>
+      <c r="H462" s="4" t="n"/>
     </row>
     <row r="463">
       <c r="A463" s="4" t="n"/>
@@ -4769,6 +5240,7 @@
       <c r="E463" s="4" t="n"/>
       <c r="F463" s="4" t="n"/>
       <c r="G463" s="4" t="n"/>
+      <c r="H463" s="4" t="n"/>
     </row>
     <row r="464">
       <c r="A464" s="4" t="n"/>
@@ -4778,6 +5250,7 @@
       <c r="E464" s="4" t="n"/>
       <c r="F464" s="4" t="n"/>
       <c r="G464" s="4" t="n"/>
+      <c r="H464" s="4" t="n"/>
     </row>
     <row r="465">
       <c r="A465" s="4" t="n"/>
@@ -4787,6 +5260,7 @@
       <c r="E465" s="4" t="n"/>
       <c r="F465" s="4" t="n"/>
       <c r="G465" s="4" t="n"/>
+      <c r="H465" s="4" t="n"/>
     </row>
     <row r="466">
       <c r="A466" s="4" t="n"/>
@@ -4796,6 +5270,7 @@
       <c r="E466" s="4" t="n"/>
       <c r="F466" s="4" t="n"/>
       <c r="G466" s="4" t="n"/>
+      <c r="H466" s="4" t="n"/>
     </row>
     <row r="467">
       <c r="A467" s="4" t="n"/>
@@ -4805,6 +5280,7 @@
       <c r="E467" s="4" t="n"/>
       <c r="F467" s="4" t="n"/>
       <c r="G467" s="4" t="n"/>
+      <c r="H467" s="4" t="n"/>
     </row>
     <row r="468">
       <c r="A468" s="4" t="n"/>
@@ -4814,6 +5290,7 @@
       <c r="E468" s="4" t="n"/>
       <c r="F468" s="4" t="n"/>
       <c r="G468" s="4" t="n"/>
+      <c r="H468" s="4" t="n"/>
     </row>
     <row r="469">
       <c r="A469" s="4" t="n"/>
@@ -4823,6 +5300,7 @@
       <c r="E469" s="4" t="n"/>
       <c r="F469" s="4" t="n"/>
       <c r="G469" s="4" t="n"/>
+      <c r="H469" s="4" t="n"/>
     </row>
     <row r="470">
       <c r="A470" s="4" t="n"/>
@@ -4832,6 +5310,7 @@
       <c r="E470" s="4" t="n"/>
       <c r="F470" s="4" t="n"/>
       <c r="G470" s="4" t="n"/>
+      <c r="H470" s="4" t="n"/>
     </row>
     <row r="471">
       <c r="A471" s="4" t="n"/>
@@ -4841,6 +5320,7 @@
       <c r="E471" s="4" t="n"/>
       <c r="F471" s="4" t="n"/>
       <c r="G471" s="4" t="n"/>
+      <c r="H471" s="4" t="n"/>
     </row>
     <row r="472">
       <c r="A472" s="4" t="n"/>
@@ -4850,6 +5330,7 @@
       <c r="E472" s="4" t="n"/>
       <c r="F472" s="4" t="n"/>
       <c r="G472" s="4" t="n"/>
+      <c r="H472" s="4" t="n"/>
     </row>
     <row r="473">
       <c r="A473" s="4" t="n"/>
@@ -4859,6 +5340,7 @@
       <c r="E473" s="4" t="n"/>
       <c r="F473" s="4" t="n"/>
       <c r="G473" s="4" t="n"/>
+      <c r="H473" s="4" t="n"/>
     </row>
     <row r="474">
       <c r="A474" s="4" t="n"/>
@@ -4868,6 +5350,7 @@
       <c r="E474" s="4" t="n"/>
       <c r="F474" s="4" t="n"/>
       <c r="G474" s="4" t="n"/>
+      <c r="H474" s="4" t="n"/>
     </row>
     <row r="475">
       <c r="A475" s="4" t="n"/>
@@ -4877,6 +5360,7 @@
       <c r="E475" s="4" t="n"/>
       <c r="F475" s="4" t="n"/>
       <c r="G475" s="4" t="n"/>
+      <c r="H475" s="4" t="n"/>
     </row>
     <row r="476">
       <c r="A476" s="4" t="n"/>
@@ -4886,6 +5370,7 @@
       <c r="E476" s="4" t="n"/>
       <c r="F476" s="4" t="n"/>
       <c r="G476" s="4" t="n"/>
+      <c r="H476" s="4" t="n"/>
     </row>
     <row r="477">
       <c r="A477" s="4" t="n"/>
@@ -4895,6 +5380,7 @@
       <c r="E477" s="4" t="n"/>
       <c r="F477" s="4" t="n"/>
       <c r="G477" s="4" t="n"/>
+      <c r="H477" s="4" t="n"/>
     </row>
     <row r="478">
       <c r="A478" s="4" t="n"/>
@@ -4904,6 +5390,7 @@
       <c r="E478" s="4" t="n"/>
       <c r="F478" s="4" t="n"/>
       <c r="G478" s="4" t="n"/>
+      <c r="H478" s="4" t="n"/>
     </row>
     <row r="479">
       <c r="A479" s="4" t="n"/>
@@ -4913,6 +5400,7 @@
       <c r="E479" s="4" t="n"/>
       <c r="F479" s="4" t="n"/>
       <c r="G479" s="4" t="n"/>
+      <c r="H479" s="4" t="n"/>
     </row>
     <row r="480">
       <c r="A480" s="4" t="n"/>
@@ -4922,6 +5410,7 @@
       <c r="E480" s="4" t="n"/>
       <c r="F480" s="4" t="n"/>
       <c r="G480" s="4" t="n"/>
+      <c r="H480" s="4" t="n"/>
     </row>
     <row r="481">
       <c r="A481" s="4" t="n"/>
@@ -4931,6 +5420,7 @@
       <c r="E481" s="4" t="n"/>
       <c r="F481" s="4" t="n"/>
       <c r="G481" s="4" t="n"/>
+      <c r="H481" s="4" t="n"/>
     </row>
     <row r="482">
       <c r="A482" s="4" t="n"/>
@@ -4940,6 +5430,7 @@
       <c r="E482" s="4" t="n"/>
       <c r="F482" s="4" t="n"/>
       <c r="G482" s="4" t="n"/>
+      <c r="H482" s="4" t="n"/>
     </row>
     <row r="483">
       <c r="A483" s="4" t="n"/>
@@ -4949,6 +5440,7 @@
       <c r="E483" s="4" t="n"/>
       <c r="F483" s="4" t="n"/>
       <c r="G483" s="4" t="n"/>
+      <c r="H483" s="4" t="n"/>
     </row>
     <row r="484">
       <c r="A484" s="4" t="n"/>
@@ -4958,6 +5450,7 @@
       <c r="E484" s="4" t="n"/>
       <c r="F484" s="4" t="n"/>
       <c r="G484" s="4" t="n"/>
+      <c r="H484" s="4" t="n"/>
     </row>
     <row r="485">
       <c r="A485" s="4" t="n"/>
@@ -4967,6 +5460,7 @@
       <c r="E485" s="4" t="n"/>
       <c r="F485" s="4" t="n"/>
       <c r="G485" s="4" t="n"/>
+      <c r="H485" s="4" t="n"/>
     </row>
     <row r="486">
       <c r="A486" s="4" t="n"/>
@@ -4976,6 +5470,7 @@
       <c r="E486" s="4" t="n"/>
       <c r="F486" s="4" t="n"/>
       <c r="G486" s="4" t="n"/>
+      <c r="H486" s="4" t="n"/>
     </row>
     <row r="487">
       <c r="A487" s="4" t="n"/>
@@ -4985,6 +5480,7 @@
       <c r="E487" s="4" t="n"/>
       <c r="F487" s="4" t="n"/>
       <c r="G487" s="4" t="n"/>
+      <c r="H487" s="4" t="n"/>
     </row>
     <row r="488">
       <c r="A488" s="4" t="n"/>
@@ -4994,6 +5490,7 @@
       <c r="E488" s="4" t="n"/>
       <c r="F488" s="4" t="n"/>
       <c r="G488" s="4" t="n"/>
+      <c r="H488" s="4" t="n"/>
     </row>
     <row r="489">
       <c r="A489" s="4" t="n"/>
@@ -5003,6 +5500,7 @@
       <c r="E489" s="4" t="n"/>
       <c r="F489" s="4" t="n"/>
       <c r="G489" s="4" t="n"/>
+      <c r="H489" s="4" t="n"/>
     </row>
     <row r="490">
       <c r="A490" s="4" t="n"/>
@@ -5012,6 +5510,7 @@
       <c r="E490" s="4" t="n"/>
       <c r="F490" s="4" t="n"/>
       <c r="G490" s="4" t="n"/>
+      <c r="H490" s="4" t="n"/>
     </row>
     <row r="491">
       <c r="A491" s="4" t="n"/>
@@ -5021,6 +5520,7 @@
       <c r="E491" s="4" t="n"/>
       <c r="F491" s="4" t="n"/>
       <c r="G491" s="4" t="n"/>
+      <c r="H491" s="4" t="n"/>
     </row>
     <row r="492">
       <c r="A492" s="4" t="n"/>
@@ -5030,6 +5530,7 @@
       <c r="E492" s="4" t="n"/>
       <c r="F492" s="4" t="n"/>
       <c r="G492" s="4" t="n"/>
+      <c r="H492" s="4" t="n"/>
     </row>
     <row r="493">
       <c r="A493" s="4" t="n"/>
@@ -5039,6 +5540,7 @@
       <c r="E493" s="4" t="n"/>
       <c r="F493" s="4" t="n"/>
       <c r="G493" s="4" t="n"/>
+      <c r="H493" s="4" t="n"/>
     </row>
     <row r="494">
       <c r="A494" s="4" t="n"/>
@@ -5048,6 +5550,7 @@
       <c r="E494" s="4" t="n"/>
       <c r="F494" s="4" t="n"/>
       <c r="G494" s="4" t="n"/>
+      <c r="H494" s="4" t="n"/>
     </row>
     <row r="495">
       <c r="A495" s="4" t="n"/>
@@ -5057,6 +5560,7 @@
       <c r="E495" s="4" t="n"/>
       <c r="F495" s="4" t="n"/>
       <c r="G495" s="4" t="n"/>
+      <c r="H495" s="4" t="n"/>
     </row>
     <row r="496">
       <c r="A496" s="4" t="n"/>
@@ -5066,6 +5570,7 @@
       <c r="E496" s="4" t="n"/>
       <c r="F496" s="4" t="n"/>
       <c r="G496" s="4" t="n"/>
+      <c r="H496" s="4" t="n"/>
     </row>
     <row r="497">
       <c r="A497" s="4" t="n"/>
@@ -5075,6 +5580,7 @@
       <c r="E497" s="4" t="n"/>
       <c r="F497" s="4" t="n"/>
       <c r="G497" s="4" t="n"/>
+      <c r="H497" s="4" t="n"/>
     </row>
     <row r="498">
       <c r="A498" s="4" t="n"/>
@@ -5084,6 +5590,7 @@
       <c r="E498" s="4" t="n"/>
       <c r="F498" s="4" t="n"/>
       <c r="G498" s="4" t="n"/>
+      <c r="H498" s="4" t="n"/>
     </row>
     <row r="499">
       <c r="A499" s="4" t="n"/>
@@ -5093,6 +5600,7 @@
       <c r="E499" s="4" t="n"/>
       <c r="F499" s="4" t="n"/>
       <c r="G499" s="4" t="n"/>
+      <c r="H499" s="4" t="n"/>
     </row>
     <row r="500">
       <c r="A500" s="4" t="n"/>
@@ -5102,6 +5610,7 @@
       <c r="E500" s="4" t="n"/>
       <c r="F500" s="4" t="n"/>
       <c r="G500" s="4" t="n"/>
+      <c r="H500" s="4" t="n"/>
     </row>
     <row r="501">
       <c r="A501" s="4" t="n"/>
@@ -5111,6 +5620,7 @@
       <c r="E501" s="4" t="n"/>
       <c r="F501" s="4" t="n"/>
       <c r="G501" s="4" t="n"/>
+      <c r="H501" s="4" t="n"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="0" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="0" insertColumns="0" pivotTables="1" deleteRows="0" formatCells="0" formatRows="0" sort="0"/>
@@ -5133,7 +5643,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5143,6 +5653,7 @@
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
     <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5245,131 +5756,155 @@
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="8" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>Party Size</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>Optional. Total people including the guest (3 = guest + 2). Seated together at the same table, checked in together.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>Example (how a row looks — do not copy this row into the Guests sheet unless it is a real guest)</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="11" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="11" t="inlineStr">
         <is>
           <t>First Name</t>
         </is>
       </c>
-      <c r="B13" s="11" t="inlineStr">
+      <c r="B14" s="11" t="inlineStr">
         <is>
           <t>Last Name</t>
         </is>
       </c>
-      <c r="C13" s="12" t="inlineStr">
+      <c r="C14" s="12" t="inlineStr">
         <is>
           <t>Table</t>
         </is>
       </c>
-      <c r="D13" s="12" t="inlineStr">
+      <c r="D14" s="12" t="inlineStr">
         <is>
           <t>Meal</t>
         </is>
       </c>
-      <c r="E13" s="12" t="inlineStr">
+      <c r="E14" s="12" t="inlineStr">
         <is>
           <t>Allergy</t>
         </is>
       </c>
-      <c r="F13" s="12" t="inlineStr">
+      <c r="F14" s="12" t="inlineStr">
         <is>
           <t>VIP</t>
         </is>
       </c>
-      <c r="G13" s="12" t="inlineStr">
+      <c r="G14" s="12" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="13" t="inlineStr">
+      <c r="H14" s="12" t="inlineStr">
+        <is>
+          <t>Party Size</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="13" t="inlineStr">
         <is>
           <t>Jodel</t>
         </is>
       </c>
-      <c r="B14" s="13" t="inlineStr">
+      <c r="B15" s="13" t="inlineStr">
         <is>
           <t>Aristilde</t>
         </is>
       </c>
-      <c r="C14" s="13" t="inlineStr">
+      <c r="C15" s="13" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="D14" s="13" t="inlineStr">
+      <c r="D15" s="13" t="inlineStr">
         <is>
           <t>Chicken</t>
         </is>
       </c>
-      <c r="E14" s="13" t="inlineStr"/>
-      <c r="F14" s="13" t="inlineStr"/>
-      <c r="G14" s="13" t="inlineStr">
+      <c r="E15" s="13" t="inlineStr"/>
+      <c r="F15" s="13" t="inlineStr"/>
+      <c r="G15" s="13" t="inlineStr">
         <is>
           <t>$250 to pay before seating</t>
         </is>
       </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="13" t="inlineStr">
+      <c r="H15" s="13" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="13" t="inlineStr">
         <is>
           <t>Marie</t>
         </is>
       </c>
-      <c r="B15" s="13" t="inlineStr">
+      <c r="B16" s="13" t="inlineStr">
         <is>
           <t>Delva</t>
         </is>
       </c>
-      <c r="C15" s="13" t="inlineStr">
+      <c r="C16" s="13" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="D15" s="13" t="inlineStr">
+      <c r="D16" s="13" t="inlineStr">
         <is>
           <t>Fish</t>
         </is>
       </c>
-      <c r="E15" s="13" t="inlineStr">
+      <c r="E16" s="13" t="inlineStr">
         <is>
           <t>Nuts</t>
         </is>
       </c>
-      <c r="F15" s="13" t="inlineStr">
+      <c r="F16" s="13" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="G15" s="13" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="13" t="inlineStr">
+      <c r="G16" s="13" t="inlineStr"/>
+      <c r="H16" s="13" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="13" t="inlineStr">
         <is>
           <t>Paul</t>
         </is>
       </c>
-      <c r="B16" s="13" t="inlineStr">
+      <c r="B17" s="13" t="inlineStr">
         <is>
           <t>Murphy</t>
         </is>
       </c>
-      <c r="C16" s="13" t="inlineStr"/>
-      <c r="D16" s="13" t="inlineStr"/>
-      <c r="E16" s="13" t="inlineStr"/>
-      <c r="F16" s="13" t="inlineStr"/>
-      <c r="G16" s="13" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="14" t="inlineStr">
+      <c r="C17" s="13" t="inlineStr"/>
+      <c r="D17" s="13" t="inlineStr"/>
+      <c r="E17" s="13" t="inlineStr"/>
+      <c r="F17" s="13" t="inlineStr"/>
+      <c r="G17" s="13" t="inlineStr"/>
+      <c r="H17" s="13" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="14" t="inlineStr">
         <is>
           <t>Tips: keep the first row of the Guests sheet as it is (the column names). Empty cells are fine. Already uploaded your guests? Use Import Guests → Update meals / allergies with the same columns to add meals, allergies, VIP or notes later.</t>
         </is>

</xml_diff>